<commit_message>
Added all files updated
</commit_message>
<xml_diff>
--- a/program_validation/Program Validation Planning Tool.xlsx
+++ b/program_validation/Program Validation Planning Tool.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20325"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jay\Downloads\FALL2017\ExcelParsing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jay\Downloads\ExcelParsing\program_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46136564-62C1-4FB6-8DD1-54FB3CFC05B8}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8859807-CA5E-40F3-81B0-A097E109486B}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="456" windowWidth="25596" windowHeight="14316" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="456" windowWidth="25596" windowHeight="14316" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,20 @@
     <sheet name="format" sheetId="2" r:id="rId3"/>
     <sheet name="Desired Format" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="179021"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1412" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1420" uniqueCount="143">
   <si>
     <t>Activity ID</t>
   </si>
@@ -865,37 +873,25 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="29" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -910,31 +906,16 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="31" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -943,19 +924,46 @@
     <xf numFmtId="0" fontId="0" fillId="31" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2206,7 +2214,9 @@
       </c>
     </row>
     <row r="64" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A64" s="24"/>
+      <c r="A64" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="B64" s="24" t="s">
         <v>78</v>
       </c>
@@ -2246,7 +2256,9 @@
       </c>
     </row>
     <row r="67" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A67" s="24"/>
+      <c r="A67" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="B67" s="24" t="s">
         <v>82</v>
       </c>
@@ -2286,7 +2298,9 @@
       </c>
     </row>
     <row r="70" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A70" s="24"/>
+      <c r="A70" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="B70" s="24" t="s">
         <v>85</v>
       </c>
@@ -2326,7 +2340,9 @@
       </c>
     </row>
     <row r="73" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A73" s="24"/>
+      <c r="A73" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="B73" s="24" t="s">
         <v>88</v>
       </c>
@@ -2366,7 +2382,9 @@
       </c>
     </row>
     <row r="76" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A76" s="24"/>
+      <c r="A76" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="B76" s="24" t="s">
         <v>91</v>
       </c>
@@ -2474,7 +2492,9 @@
       </c>
     </row>
     <row r="84" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A84" s="24"/>
+      <c r="A84" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="B84" s="24" t="s">
         <v>99</v>
       </c>
@@ -2514,7 +2534,9 @@
       </c>
     </row>
     <row r="87" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A87" s="24"/>
+      <c r="A87" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="B87" s="24" t="s">
         <v>103</v>
       </c>
@@ -2554,7 +2576,9 @@
       </c>
     </row>
     <row r="90" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A90" s="24"/>
+      <c r="A90" s="24" t="s">
+        <v>4</v>
+      </c>
       <c r="B90" s="24" t="s">
         <v>106</v>
       </c>
@@ -6235,9 +6259,7 @@
   <cols>
     <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" customWidth="1"/>
+    <col min="3" max="9" width="6.5546875" customWidth="1"/>
     <col min="11" max="11" width="10.77734375" customWidth="1"/>
     <col min="129" max="129" width="15.77734375" bestFit="1" customWidth="1"/>
     <col min="130" max="130" width="24" bestFit="1" customWidth="1"/>
@@ -6307,951 +6329,951 @@
       <c r="B1" t="s">
         <v>126</v>
       </c>
-      <c r="C1" s="63">
+      <c r="C1" s="39">
         <v>43101</v>
       </c>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63">
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39">
         <v>43108</v>
       </c>
-      <c r="K1" s="63"/>
-      <c r="L1" s="63"/>
-      <c r="M1" s="63"/>
-      <c r="N1" s="63"/>
-      <c r="O1" s="63"/>
-      <c r="P1" s="63"/>
-      <c r="Q1" s="63">
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39">
         <v>43115</v>
       </c>
-      <c r="R1" s="63"/>
-      <c r="S1" s="63"/>
-      <c r="T1" s="63"/>
-      <c r="U1" s="63"/>
-      <c r="V1" s="63"/>
-      <c r="W1" s="63"/>
-      <c r="X1" s="63">
+      <c r="R1" s="39"/>
+      <c r="S1" s="39"/>
+      <c r="T1" s="39"/>
+      <c r="U1" s="39"/>
+      <c r="V1" s="39"/>
+      <c r="W1" s="39"/>
+      <c r="X1" s="39">
         <v>43122</v>
       </c>
-      <c r="Y1" s="63"/>
-      <c r="Z1" s="63"/>
-      <c r="AA1" s="63"/>
-      <c r="AB1" s="63"/>
-      <c r="AC1" s="63"/>
-      <c r="AD1" s="63"/>
-      <c r="AE1" s="63">
+      <c r="Y1" s="39"/>
+      <c r="Z1" s="39"/>
+      <c r="AA1" s="39"/>
+      <c r="AB1" s="39"/>
+      <c r="AC1" s="39"/>
+      <c r="AD1" s="39"/>
+      <c r="AE1" s="39">
         <v>43129</v>
       </c>
-      <c r="AF1" s="63"/>
-      <c r="AG1" s="63"/>
-      <c r="AH1" s="63"/>
-      <c r="AI1" s="63"/>
-      <c r="AJ1" s="63"/>
-      <c r="AK1" s="63"/>
-      <c r="AL1" s="63">
+      <c r="AF1" s="39"/>
+      <c r="AG1" s="39"/>
+      <c r="AH1" s="39"/>
+      <c r="AI1" s="39"/>
+      <c r="AJ1" s="39"/>
+      <c r="AK1" s="39"/>
+      <c r="AL1" s="39">
         <v>43136</v>
       </c>
-      <c r="AM1" s="63"/>
-      <c r="AN1" s="63"/>
-      <c r="AO1" s="63"/>
-      <c r="AP1" s="63"/>
-      <c r="AQ1" s="63"/>
-      <c r="AR1" s="63"/>
-      <c r="AS1" s="63">
+      <c r="AM1" s="39"/>
+      <c r="AN1" s="39"/>
+      <c r="AO1" s="39"/>
+      <c r="AP1" s="39"/>
+      <c r="AQ1" s="39"/>
+      <c r="AR1" s="39"/>
+      <c r="AS1" s="39">
         <v>43143</v>
       </c>
-      <c r="AT1" s="63"/>
-      <c r="AU1" s="63"/>
-      <c r="AV1" s="63"/>
-      <c r="AW1" s="63"/>
-      <c r="AX1" s="63"/>
-      <c r="AY1" s="63"/>
-      <c r="AZ1" s="63">
+      <c r="AT1" s="39"/>
+      <c r="AU1" s="39"/>
+      <c r="AV1" s="39"/>
+      <c r="AW1" s="39"/>
+      <c r="AX1" s="39"/>
+      <c r="AY1" s="39"/>
+      <c r="AZ1" s="39">
         <v>43150</v>
       </c>
-      <c r="BA1" s="63"/>
-      <c r="BB1" s="63"/>
-      <c r="BC1" s="63"/>
-      <c r="BD1" s="63"/>
-      <c r="BE1" s="63"/>
-      <c r="BF1" s="63"/>
-      <c r="BG1" s="63">
+      <c r="BA1" s="39"/>
+      <c r="BB1" s="39"/>
+      <c r="BC1" s="39"/>
+      <c r="BD1" s="39"/>
+      <c r="BE1" s="39"/>
+      <c r="BF1" s="39"/>
+      <c r="BG1" s="39">
         <v>43157</v>
       </c>
-      <c r="BH1" s="63"/>
-      <c r="BI1" s="63"/>
-      <c r="BJ1" s="63"/>
-      <c r="BK1" s="63"/>
-      <c r="BL1" s="63"/>
-      <c r="BM1" s="63"/>
-      <c r="BN1" s="63">
+      <c r="BH1" s="39"/>
+      <c r="BI1" s="39"/>
+      <c r="BJ1" s="39"/>
+      <c r="BK1" s="39"/>
+      <c r="BL1" s="39"/>
+      <c r="BM1" s="39"/>
+      <c r="BN1" s="39">
         <v>43164</v>
       </c>
-      <c r="BO1" s="63"/>
-      <c r="BP1" s="63"/>
-      <c r="BQ1" s="63"/>
-      <c r="BR1" s="63"/>
-      <c r="BS1" s="63"/>
-      <c r="BT1" s="63"/>
-      <c r="BU1" s="63">
+      <c r="BO1" s="39"/>
+      <c r="BP1" s="39"/>
+      <c r="BQ1" s="39"/>
+      <c r="BR1" s="39"/>
+      <c r="BS1" s="39"/>
+      <c r="BT1" s="39"/>
+      <c r="BU1" s="39">
         <v>43171</v>
       </c>
-      <c r="BV1" s="63"/>
-      <c r="BW1" s="63"/>
-      <c r="BX1" s="63"/>
-      <c r="BY1" s="63"/>
-      <c r="BZ1" s="63"/>
-      <c r="CA1" s="63"/>
-      <c r="CB1" s="63">
+      <c r="BV1" s="39"/>
+      <c r="BW1" s="39"/>
+      <c r="BX1" s="39"/>
+      <c r="BY1" s="39"/>
+      <c r="BZ1" s="39"/>
+      <c r="CA1" s="39"/>
+      <c r="CB1" s="39">
         <v>43178</v>
       </c>
-      <c r="CC1" s="63"/>
-      <c r="CD1" s="63"/>
-      <c r="CE1" s="63"/>
-      <c r="CF1" s="63"/>
-      <c r="CG1" s="63"/>
-      <c r="CH1" s="63"/>
-      <c r="CI1" s="63">
+      <c r="CC1" s="39"/>
+      <c r="CD1" s="39"/>
+      <c r="CE1" s="39"/>
+      <c r="CF1" s="39"/>
+      <c r="CG1" s="39"/>
+      <c r="CH1" s="39"/>
+      <c r="CI1" s="39">
         <v>43185</v>
       </c>
-      <c r="CJ1" s="63"/>
-      <c r="CK1" s="63"/>
-      <c r="CL1" s="63"/>
-      <c r="CM1" s="63"/>
-      <c r="CN1" s="63"/>
-      <c r="CO1" s="63"/>
-      <c r="CP1" s="63">
+      <c r="CJ1" s="39"/>
+      <c r="CK1" s="39"/>
+      <c r="CL1" s="39"/>
+      <c r="CM1" s="39"/>
+      <c r="CN1" s="39"/>
+      <c r="CO1" s="39"/>
+      <c r="CP1" s="39">
         <v>43192</v>
       </c>
-      <c r="CQ1" s="63"/>
-      <c r="CR1" s="63"/>
-      <c r="CS1" s="63"/>
-      <c r="CT1" s="63"/>
-      <c r="CU1" s="63"/>
-      <c r="CV1" s="63"/>
-      <c r="CW1" s="63">
+      <c r="CQ1" s="39"/>
+      <c r="CR1" s="39"/>
+      <c r="CS1" s="39"/>
+      <c r="CT1" s="39"/>
+      <c r="CU1" s="39"/>
+      <c r="CV1" s="39"/>
+      <c r="CW1" s="39">
         <v>43199</v>
       </c>
-      <c r="CX1" s="63"/>
-      <c r="CY1" s="63"/>
-      <c r="CZ1" s="63"/>
-      <c r="DA1" s="63"/>
-      <c r="DB1" s="63"/>
-      <c r="DC1" s="63"/>
-      <c r="DD1" s="63">
+      <c r="CX1" s="39"/>
+      <c r="CY1" s="39"/>
+      <c r="CZ1" s="39"/>
+      <c r="DA1" s="39"/>
+      <c r="DB1" s="39"/>
+      <c r="DC1" s="39"/>
+      <c r="DD1" s="39">
         <v>43206</v>
       </c>
-      <c r="DE1" s="63"/>
-      <c r="DF1" s="63"/>
-      <c r="DG1" s="63"/>
-      <c r="DH1" s="63"/>
-      <c r="DI1" s="63"/>
-      <c r="DJ1" s="63"/>
-      <c r="DK1" s="63">
+      <c r="DE1" s="39"/>
+      <c r="DF1" s="39"/>
+      <c r="DG1" s="39"/>
+      <c r="DH1" s="39"/>
+      <c r="DI1" s="39"/>
+      <c r="DJ1" s="39"/>
+      <c r="DK1" s="39">
         <v>43213</v>
       </c>
-      <c r="DL1" s="63"/>
-      <c r="DM1" s="63"/>
-      <c r="DN1" s="63"/>
-      <c r="DO1" s="63"/>
-      <c r="DP1" s="63"/>
-      <c r="DQ1" s="63"/>
-      <c r="DR1" s="63">
+      <c r="DL1" s="39"/>
+      <c r="DM1" s="39"/>
+      <c r="DN1" s="39"/>
+      <c r="DO1" s="39"/>
+      <c r="DP1" s="39"/>
+      <c r="DQ1" s="39"/>
+      <c r="DR1" s="39">
         <v>43220</v>
       </c>
-      <c r="DS1" s="63"/>
-      <c r="DT1" s="63"/>
-      <c r="DU1" s="63"/>
-      <c r="DV1" s="63"/>
-      <c r="DW1" s="63"/>
-      <c r="DX1" s="63"/>
-      <c r="DY1" s="63">
+      <c r="DS1" s="39"/>
+      <c r="DT1" s="39"/>
+      <c r="DU1" s="39"/>
+      <c r="DV1" s="39"/>
+      <c r="DW1" s="39"/>
+      <c r="DX1" s="39"/>
+      <c r="DY1" s="39">
         <v>43227</v>
       </c>
-      <c r="DZ1" s="63"/>
-      <c r="EA1" s="63"/>
-      <c r="EB1" s="63"/>
-      <c r="EC1" s="63"/>
-      <c r="ED1" s="63"/>
-      <c r="EE1" s="63"/>
-      <c r="EF1" s="63">
+      <c r="DZ1" s="39"/>
+      <c r="EA1" s="39"/>
+      <c r="EB1" s="39"/>
+      <c r="EC1" s="39"/>
+      <c r="ED1" s="39"/>
+      <c r="EE1" s="39"/>
+      <c r="EF1" s="39">
         <v>43234</v>
       </c>
-      <c r="EG1" s="63"/>
-      <c r="EH1" s="63"/>
-      <c r="EI1" s="63"/>
-      <c r="EJ1" s="63"/>
-      <c r="EK1" s="63"/>
-      <c r="EL1" s="63"/>
-      <c r="EM1" s="63">
+      <c r="EG1" s="39"/>
+      <c r="EH1" s="39"/>
+      <c r="EI1" s="39"/>
+      <c r="EJ1" s="39"/>
+      <c r="EK1" s="39"/>
+      <c r="EL1" s="39"/>
+      <c r="EM1" s="39">
         <v>43241</v>
       </c>
-      <c r="EN1" s="63"/>
-      <c r="EO1" s="63"/>
-      <c r="EP1" s="63"/>
-      <c r="EQ1" s="63"/>
-      <c r="ER1" s="63"/>
-      <c r="ES1" s="63"/>
-      <c r="ET1" s="63">
+      <c r="EN1" s="39"/>
+      <c r="EO1" s="39"/>
+      <c r="EP1" s="39"/>
+      <c r="EQ1" s="39"/>
+      <c r="ER1" s="39"/>
+      <c r="ES1" s="39"/>
+      <c r="ET1" s="39">
         <v>43248</v>
       </c>
-      <c r="EU1" s="63"/>
-      <c r="EV1" s="63"/>
-      <c r="EW1" s="63"/>
-      <c r="EX1" s="63"/>
-      <c r="EY1" s="63"/>
-      <c r="EZ1" s="63"/>
-      <c r="FA1" s="63">
+      <c r="EU1" s="39"/>
+      <c r="EV1" s="39"/>
+      <c r="EW1" s="39"/>
+      <c r="EX1" s="39"/>
+      <c r="EY1" s="39"/>
+      <c r="EZ1" s="39"/>
+      <c r="FA1" s="39">
         <v>43255</v>
       </c>
-      <c r="FB1" s="63"/>
-      <c r="FC1" s="63"/>
-      <c r="FD1" s="63"/>
-      <c r="FE1" s="63"/>
-      <c r="FF1" s="63"/>
-      <c r="FG1" s="63"/>
-      <c r="FH1" s="63">
+      <c r="FB1" s="39"/>
+      <c r="FC1" s="39"/>
+      <c r="FD1" s="39"/>
+      <c r="FE1" s="39"/>
+      <c r="FF1" s="39"/>
+      <c r="FG1" s="39"/>
+      <c r="FH1" s="39">
         <v>43262</v>
       </c>
-      <c r="FI1" s="63"/>
-      <c r="FJ1" s="63"/>
-      <c r="FK1" s="63"/>
-      <c r="FL1" s="63"/>
-      <c r="FM1" s="63"/>
-      <c r="FN1" s="63"/>
-      <c r="FO1" s="63">
+      <c r="FI1" s="39"/>
+      <c r="FJ1" s="39"/>
+      <c r="FK1" s="39"/>
+      <c r="FL1" s="39"/>
+      <c r="FM1" s="39"/>
+      <c r="FN1" s="39"/>
+      <c r="FO1" s="39">
         <v>43269</v>
       </c>
-      <c r="FP1" s="63"/>
-      <c r="FQ1" s="63"/>
-      <c r="FR1" s="63"/>
-      <c r="FS1" s="63"/>
-      <c r="FT1" s="63"/>
-      <c r="FU1" s="63"/>
-      <c r="FV1" s="63">
+      <c r="FP1" s="39"/>
+      <c r="FQ1" s="39"/>
+      <c r="FR1" s="39"/>
+      <c r="FS1" s="39"/>
+      <c r="FT1" s="39"/>
+      <c r="FU1" s="39"/>
+      <c r="FV1" s="39">
         <v>43276</v>
       </c>
-      <c r="FW1" s="63"/>
-      <c r="FX1" s="63"/>
-      <c r="FY1" s="63"/>
-      <c r="FZ1" s="63"/>
-      <c r="GA1" s="63"/>
-      <c r="GB1" s="63"/>
-      <c r="GC1" s="63">
+      <c r="FW1" s="39"/>
+      <c r="FX1" s="39"/>
+      <c r="FY1" s="39"/>
+      <c r="FZ1" s="39"/>
+      <c r="GA1" s="39"/>
+      <c r="GB1" s="39"/>
+      <c r="GC1" s="39">
         <v>43283</v>
       </c>
-      <c r="GD1" s="63"/>
-      <c r="GE1" s="63"/>
-      <c r="GF1" s="63"/>
-      <c r="GG1" s="63"/>
-      <c r="GH1" s="63"/>
-      <c r="GI1" s="63"/>
-      <c r="GJ1" s="63">
+      <c r="GD1" s="39"/>
+      <c r="GE1" s="39"/>
+      <c r="GF1" s="39"/>
+      <c r="GG1" s="39"/>
+      <c r="GH1" s="39"/>
+      <c r="GI1" s="39"/>
+      <c r="GJ1" s="39">
         <v>43290</v>
       </c>
-      <c r="GK1" s="63"/>
-      <c r="GL1" s="63"/>
-      <c r="GM1" s="63"/>
-      <c r="GN1" s="63"/>
-      <c r="GO1" s="63"/>
-      <c r="GP1" s="63"/>
-      <c r="GQ1" s="63">
+      <c r="GK1" s="39"/>
+      <c r="GL1" s="39"/>
+      <c r="GM1" s="39"/>
+      <c r="GN1" s="39"/>
+      <c r="GO1" s="39"/>
+      <c r="GP1" s="39"/>
+      <c r="GQ1" s="39">
         <v>43297</v>
       </c>
-      <c r="GR1" s="63"/>
-      <c r="GS1" s="63"/>
-      <c r="GT1" s="63"/>
-      <c r="GU1" s="63"/>
-      <c r="GV1" s="63"/>
-      <c r="GW1" s="63"/>
-      <c r="GX1" s="63">
+      <c r="GR1" s="39"/>
+      <c r="GS1" s="39"/>
+      <c r="GT1" s="39"/>
+      <c r="GU1" s="39"/>
+      <c r="GV1" s="39"/>
+      <c r="GW1" s="39"/>
+      <c r="GX1" s="39">
         <v>43304</v>
       </c>
-      <c r="GY1" s="63"/>
-      <c r="GZ1" s="63"/>
-      <c r="HA1" s="63"/>
-      <c r="HB1" s="63"/>
-      <c r="HC1" s="63"/>
-      <c r="HD1" s="63"/>
-      <c r="HE1" s="63">
+      <c r="GY1" s="39"/>
+      <c r="GZ1" s="39"/>
+      <c r="HA1" s="39"/>
+      <c r="HB1" s="39"/>
+      <c r="HC1" s="39"/>
+      <c r="HD1" s="39"/>
+      <c r="HE1" s="39">
         <v>43311</v>
       </c>
-      <c r="HF1" s="63"/>
-      <c r="HG1" s="63"/>
-      <c r="HH1" s="63"/>
-      <c r="HI1" s="63"/>
-      <c r="HJ1" s="63"/>
-      <c r="HK1" s="63"/>
-      <c r="HL1" s="63">
+      <c r="HF1" s="39"/>
+      <c r="HG1" s="39"/>
+      <c r="HH1" s="39"/>
+      <c r="HI1" s="39"/>
+      <c r="HJ1" s="39"/>
+      <c r="HK1" s="39"/>
+      <c r="HL1" s="39">
         <v>43318</v>
       </c>
-      <c r="HM1" s="63"/>
-      <c r="HN1" s="63"/>
-      <c r="HO1" s="63"/>
-      <c r="HP1" s="63"/>
-      <c r="HQ1" s="63"/>
-      <c r="HR1" s="63"/>
-      <c r="HS1" s="63">
+      <c r="HM1" s="39"/>
+      <c r="HN1" s="39"/>
+      <c r="HO1" s="39"/>
+      <c r="HP1" s="39"/>
+      <c r="HQ1" s="39"/>
+      <c r="HR1" s="39"/>
+      <c r="HS1" s="39">
         <v>43325</v>
       </c>
-      <c r="HT1" s="63"/>
-      <c r="HU1" s="63"/>
-      <c r="HV1" s="63"/>
-      <c r="HW1" s="63"/>
-      <c r="HX1" s="63"/>
-      <c r="HY1" s="63"/>
-      <c r="HZ1" s="63">
+      <c r="HT1" s="39"/>
+      <c r="HU1" s="39"/>
+      <c r="HV1" s="39"/>
+      <c r="HW1" s="39"/>
+      <c r="HX1" s="39"/>
+      <c r="HY1" s="39"/>
+      <c r="HZ1" s="39">
         <v>43332</v>
       </c>
-      <c r="IA1" s="63"/>
-      <c r="IB1" s="63"/>
-      <c r="IC1" s="63"/>
-      <c r="ID1" s="63"/>
-      <c r="IE1" s="63"/>
-      <c r="IF1" s="63"/>
-      <c r="IG1" s="63">
+      <c r="IA1" s="39"/>
+      <c r="IB1" s="39"/>
+      <c r="IC1" s="39"/>
+      <c r="ID1" s="39"/>
+      <c r="IE1" s="39"/>
+      <c r="IF1" s="39"/>
+      <c r="IG1" s="39">
         <v>43339</v>
       </c>
-      <c r="IH1" s="63"/>
-      <c r="II1" s="63"/>
-      <c r="IJ1" s="63"/>
-      <c r="IK1" s="63"/>
-      <c r="IL1" s="63"/>
-      <c r="IM1" s="63"/>
-      <c r="IN1" s="63">
+      <c r="IH1" s="39"/>
+      <c r="II1" s="39"/>
+      <c r="IJ1" s="39"/>
+      <c r="IK1" s="39"/>
+      <c r="IL1" s="39"/>
+      <c r="IM1" s="39"/>
+      <c r="IN1" s="39">
         <v>43346</v>
       </c>
-      <c r="IO1" s="63"/>
-      <c r="IP1" s="63"/>
-      <c r="IQ1" s="63"/>
-      <c r="IR1" s="63"/>
-      <c r="IS1" s="63"/>
-      <c r="IT1" s="63"/>
-      <c r="IU1" s="63">
+      <c r="IO1" s="39"/>
+      <c r="IP1" s="39"/>
+      <c r="IQ1" s="39"/>
+      <c r="IR1" s="39"/>
+      <c r="IS1" s="39"/>
+      <c r="IT1" s="39"/>
+      <c r="IU1" s="39">
         <v>43353</v>
       </c>
-      <c r="IV1" s="63"/>
-      <c r="IW1" s="63"/>
-      <c r="IX1" s="63"/>
-      <c r="IY1" s="63"/>
-      <c r="IZ1" s="63"/>
-      <c r="JA1" s="63"/>
-      <c r="JB1" s="63">
+      <c r="IV1" s="39"/>
+      <c r="IW1" s="39"/>
+      <c r="IX1" s="39"/>
+      <c r="IY1" s="39"/>
+      <c r="IZ1" s="39"/>
+      <c r="JA1" s="39"/>
+      <c r="JB1" s="39">
         <v>43360</v>
       </c>
-      <c r="JC1" s="63"/>
-      <c r="JD1" s="63"/>
-      <c r="JE1" s="63"/>
-      <c r="JF1" s="63"/>
-      <c r="JG1" s="63"/>
-      <c r="JH1" s="63"/>
-      <c r="JI1" s="63">
+      <c r="JC1" s="39"/>
+      <c r="JD1" s="39"/>
+      <c r="JE1" s="39"/>
+      <c r="JF1" s="39"/>
+      <c r="JG1" s="39"/>
+      <c r="JH1" s="39"/>
+      <c r="JI1" s="39">
         <v>43367</v>
       </c>
-      <c r="JJ1" s="63"/>
-      <c r="JK1" s="63"/>
-      <c r="JL1" s="63"/>
-      <c r="JM1" s="63"/>
-      <c r="JN1" s="63"/>
-      <c r="JO1" s="63"/>
-      <c r="JP1" s="63">
+      <c r="JJ1" s="39"/>
+      <c r="JK1" s="39"/>
+      <c r="JL1" s="39"/>
+      <c r="JM1" s="39"/>
+      <c r="JN1" s="39"/>
+      <c r="JO1" s="39"/>
+      <c r="JP1" s="39">
         <v>43374</v>
       </c>
-      <c r="JQ1" s="63"/>
-      <c r="JR1" s="63"/>
-      <c r="JS1" s="63"/>
-      <c r="JT1" s="63"/>
-      <c r="JU1" s="63"/>
-      <c r="JV1" s="63"/>
-      <c r="JW1" s="63">
+      <c r="JQ1" s="39"/>
+      <c r="JR1" s="39"/>
+      <c r="JS1" s="39"/>
+      <c r="JT1" s="39"/>
+      <c r="JU1" s="39"/>
+      <c r="JV1" s="39"/>
+      <c r="JW1" s="39">
         <v>43381</v>
       </c>
-      <c r="JX1" s="63"/>
-      <c r="JY1" s="63"/>
-      <c r="JZ1" s="63"/>
-      <c r="KA1" s="63"/>
-      <c r="KB1" s="63"/>
-      <c r="KC1" s="63"/>
-      <c r="KD1" s="63">
+      <c r="JX1" s="39"/>
+      <c r="JY1" s="39"/>
+      <c r="JZ1" s="39"/>
+      <c r="KA1" s="39"/>
+      <c r="KB1" s="39"/>
+      <c r="KC1" s="39"/>
+      <c r="KD1" s="39">
         <v>43388</v>
       </c>
-      <c r="KE1" s="63"/>
-      <c r="KF1" s="63"/>
-      <c r="KG1" s="63"/>
-      <c r="KH1" s="63"/>
-      <c r="KI1" s="63"/>
-      <c r="KJ1" s="63"/>
-      <c r="KK1" s="63">
+      <c r="KE1" s="39"/>
+      <c r="KF1" s="39"/>
+      <c r="KG1" s="39"/>
+      <c r="KH1" s="39"/>
+      <c r="KI1" s="39"/>
+      <c r="KJ1" s="39"/>
+      <c r="KK1" s="39">
         <v>43395</v>
       </c>
-      <c r="KL1" s="63"/>
-      <c r="KM1" s="63"/>
-      <c r="KN1" s="63"/>
-      <c r="KO1" s="63"/>
-      <c r="KP1" s="63"/>
-      <c r="KQ1" s="63"/>
-      <c r="KR1" s="63">
+      <c r="KL1" s="39"/>
+      <c r="KM1" s="39"/>
+      <c r="KN1" s="39"/>
+      <c r="KO1" s="39"/>
+      <c r="KP1" s="39"/>
+      <c r="KQ1" s="39"/>
+      <c r="KR1" s="39">
         <v>43402</v>
       </c>
-      <c r="KS1" s="63"/>
-      <c r="KT1" s="63"/>
-      <c r="KU1" s="63"/>
-      <c r="KV1" s="63"/>
-      <c r="KW1" s="63"/>
-      <c r="KX1" s="63"/>
-      <c r="KY1" s="63">
+      <c r="KS1" s="39"/>
+      <c r="KT1" s="39"/>
+      <c r="KU1" s="39"/>
+      <c r="KV1" s="39"/>
+      <c r="KW1" s="39"/>
+      <c r="KX1" s="39"/>
+      <c r="KY1" s="39">
         <v>43409</v>
       </c>
-      <c r="KZ1" s="63"/>
-      <c r="LA1" s="63"/>
-      <c r="LB1" s="63"/>
-      <c r="LC1" s="63"/>
-      <c r="LD1" s="63"/>
-      <c r="LE1" s="63"/>
-      <c r="LF1" s="63">
+      <c r="KZ1" s="39"/>
+      <c r="LA1" s="39"/>
+      <c r="LB1" s="39"/>
+      <c r="LC1" s="39"/>
+      <c r="LD1" s="39"/>
+      <c r="LE1" s="39"/>
+      <c r="LF1" s="39">
         <v>43416</v>
       </c>
-      <c r="LG1" s="63"/>
-      <c r="LH1" s="63"/>
-      <c r="LI1" s="63"/>
-      <c r="LJ1" s="63"/>
-      <c r="LK1" s="63"/>
-      <c r="LL1" s="63"/>
-      <c r="LM1" s="63">
+      <c r="LG1" s="39"/>
+      <c r="LH1" s="39"/>
+      <c r="LI1" s="39"/>
+      <c r="LJ1" s="39"/>
+      <c r="LK1" s="39"/>
+      <c r="LL1" s="39"/>
+      <c r="LM1" s="39">
         <v>43423</v>
       </c>
-      <c r="LN1" s="63"/>
-      <c r="LO1" s="63"/>
-      <c r="LP1" s="63"/>
-      <c r="LQ1" s="63"/>
-      <c r="LR1" s="63"/>
-      <c r="LS1" s="63"/>
-      <c r="LT1" s="63">
+      <c r="LN1" s="39"/>
+      <c r="LO1" s="39"/>
+      <c r="LP1" s="39"/>
+      <c r="LQ1" s="39"/>
+      <c r="LR1" s="39"/>
+      <c r="LS1" s="39"/>
+      <c r="LT1" s="39">
         <v>43430</v>
       </c>
-      <c r="LU1" s="63"/>
-      <c r="LV1" s="63"/>
-      <c r="LW1" s="63"/>
-      <c r="LX1" s="63"/>
-      <c r="LY1" s="63"/>
-      <c r="LZ1" s="63"/>
-      <c r="MA1" s="63">
+      <c r="LU1" s="39"/>
+      <c r="LV1" s="39"/>
+      <c r="LW1" s="39"/>
+      <c r="LX1" s="39"/>
+      <c r="LY1" s="39"/>
+      <c r="LZ1" s="39"/>
+      <c r="MA1" s="39">
         <v>43437</v>
       </c>
-      <c r="MB1" s="63"/>
-      <c r="MC1" s="63"/>
-      <c r="MD1" s="63"/>
-      <c r="ME1" s="63"/>
-      <c r="MF1" s="63"/>
-      <c r="MG1" s="63"/>
-      <c r="MH1" s="63">
+      <c r="MB1" s="39"/>
+      <c r="MC1" s="39"/>
+      <c r="MD1" s="39"/>
+      <c r="ME1" s="39"/>
+      <c r="MF1" s="39"/>
+      <c r="MG1" s="39"/>
+      <c r="MH1" s="39">
         <v>43444</v>
       </c>
-      <c r="MI1" s="63"/>
-      <c r="MJ1" s="63"/>
-      <c r="MK1" s="63"/>
-      <c r="ML1" s="63"/>
-      <c r="MM1" s="63"/>
-      <c r="MN1" s="63"/>
-      <c r="MO1" s="63">
+      <c r="MI1" s="39"/>
+      <c r="MJ1" s="39"/>
+      <c r="MK1" s="39"/>
+      <c r="ML1" s="39"/>
+      <c r="MM1" s="39"/>
+      <c r="MN1" s="39"/>
+      <c r="MO1" s="39">
         <v>43451</v>
       </c>
-      <c r="MP1" s="63"/>
-      <c r="MQ1" s="63"/>
-      <c r="MR1" s="63"/>
-      <c r="MS1" s="63"/>
-      <c r="MT1" s="63"/>
-      <c r="MU1" s="63"/>
-      <c r="MV1" s="63">
+      <c r="MP1" s="39"/>
+      <c r="MQ1" s="39"/>
+      <c r="MR1" s="39"/>
+      <c r="MS1" s="39"/>
+      <c r="MT1" s="39"/>
+      <c r="MU1" s="39"/>
+      <c r="MV1" s="39">
         <v>43458</v>
       </c>
-      <c r="MW1" s="63"/>
-      <c r="MX1" s="63"/>
-      <c r="MY1" s="63"/>
-      <c r="MZ1" s="63"/>
-      <c r="NA1" s="63"/>
-      <c r="NB1" s="63"/>
-      <c r="NC1" s="63">
+      <c r="MW1" s="39"/>
+      <c r="MX1" s="39"/>
+      <c r="MY1" s="39"/>
+      <c r="MZ1" s="39"/>
+      <c r="NA1" s="39"/>
+      <c r="NB1" s="39"/>
+      <c r="NC1" s="39">
         <v>43465</v>
       </c>
-      <c r="ND1" s="63"/>
-      <c r="NE1" s="63"/>
-      <c r="NF1" s="63"/>
-      <c r="NG1" s="63"/>
-      <c r="NH1" s="63"/>
-      <c r="NI1" s="63"/>
-      <c r="NJ1" s="63">
+      <c r="ND1" s="39"/>
+      <c r="NE1" s="39"/>
+      <c r="NF1" s="39"/>
+      <c r="NG1" s="39"/>
+      <c r="NH1" s="39"/>
+      <c r="NI1" s="39"/>
+      <c r="NJ1" s="39">
         <v>43472</v>
       </c>
-      <c r="NK1" s="63"/>
-      <c r="NL1" s="63"/>
-      <c r="NM1" s="63"/>
-      <c r="NN1" s="63"/>
-      <c r="NO1" s="63"/>
-      <c r="NP1" s="63"/>
-      <c r="NQ1" s="63">
+      <c r="NK1" s="39"/>
+      <c r="NL1" s="39"/>
+      <c r="NM1" s="39"/>
+      <c r="NN1" s="39"/>
+      <c r="NO1" s="39"/>
+      <c r="NP1" s="39"/>
+      <c r="NQ1" s="39">
         <v>43479</v>
       </c>
-      <c r="NR1" s="63"/>
-      <c r="NS1" s="63"/>
-      <c r="NT1" s="63"/>
-      <c r="NU1" s="63"/>
-      <c r="NV1" s="63"/>
-      <c r="NW1" s="63"/>
-      <c r="NX1" s="63">
+      <c r="NR1" s="39"/>
+      <c r="NS1" s="39"/>
+      <c r="NT1" s="39"/>
+      <c r="NU1" s="39"/>
+      <c r="NV1" s="39"/>
+      <c r="NW1" s="39"/>
+      <c r="NX1" s="39">
         <v>43486</v>
       </c>
-      <c r="NY1" s="63"/>
-      <c r="NZ1" s="63"/>
-      <c r="OA1" s="63"/>
-      <c r="OB1" s="63"/>
-      <c r="OC1" s="63"/>
-      <c r="OD1" s="63"/>
-      <c r="OE1" s="63">
+      <c r="NY1" s="39"/>
+      <c r="NZ1" s="39"/>
+      <c r="OA1" s="39"/>
+      <c r="OB1" s="39"/>
+      <c r="OC1" s="39"/>
+      <c r="OD1" s="39"/>
+      <c r="OE1" s="39">
         <v>43493</v>
       </c>
-      <c r="OF1" s="63"/>
-      <c r="OG1" s="63"/>
-      <c r="OH1" s="63"/>
-      <c r="OI1" s="63"/>
-      <c r="OJ1" s="63"/>
-      <c r="OK1" s="63"/>
-      <c r="OL1" s="63">
+      <c r="OF1" s="39"/>
+      <c r="OG1" s="39"/>
+      <c r="OH1" s="39"/>
+      <c r="OI1" s="39"/>
+      <c r="OJ1" s="39"/>
+      <c r="OK1" s="39"/>
+      <c r="OL1" s="39">
         <v>43500</v>
       </c>
-      <c r="OM1" s="63"/>
-      <c r="ON1" s="63"/>
-      <c r="OO1" s="63"/>
-      <c r="OP1" s="63"/>
-      <c r="OQ1" s="63"/>
-      <c r="OR1" s="63"/>
-      <c r="OS1" s="63">
+      <c r="OM1" s="39"/>
+      <c r="ON1" s="39"/>
+      <c r="OO1" s="39"/>
+      <c r="OP1" s="39"/>
+      <c r="OQ1" s="39"/>
+      <c r="OR1" s="39"/>
+      <c r="OS1" s="39">
         <v>43507</v>
       </c>
-      <c r="OT1" s="63"/>
-      <c r="OU1" s="63"/>
-      <c r="OV1" s="63"/>
-      <c r="OW1" s="63"/>
-      <c r="OX1" s="63"/>
-      <c r="OY1" s="63"/>
-      <c r="OZ1" s="63">
+      <c r="OT1" s="39"/>
+      <c r="OU1" s="39"/>
+      <c r="OV1" s="39"/>
+      <c r="OW1" s="39"/>
+      <c r="OX1" s="39"/>
+      <c r="OY1" s="39"/>
+      <c r="OZ1" s="39">
         <v>43514</v>
       </c>
-      <c r="PA1" s="63"/>
-      <c r="PB1" s="63"/>
-      <c r="PC1" s="63"/>
-      <c r="PD1" s="63"/>
-      <c r="PE1" s="63"/>
-      <c r="PF1" s="63"/>
-      <c r="PG1" s="63">
+      <c r="PA1" s="39"/>
+      <c r="PB1" s="39"/>
+      <c r="PC1" s="39"/>
+      <c r="PD1" s="39"/>
+      <c r="PE1" s="39"/>
+      <c r="PF1" s="39"/>
+      <c r="PG1" s="39">
         <v>43521</v>
       </c>
-      <c r="PH1" s="63"/>
-      <c r="PI1" s="63"/>
-      <c r="PJ1" s="63"/>
-      <c r="PK1" s="63"/>
-      <c r="PL1" s="63"/>
-      <c r="PM1" s="63"/>
-      <c r="PN1" s="63">
+      <c r="PH1" s="39"/>
+      <c r="PI1" s="39"/>
+      <c r="PJ1" s="39"/>
+      <c r="PK1" s="39"/>
+      <c r="PL1" s="39"/>
+      <c r="PM1" s="39"/>
+      <c r="PN1" s="39">
         <v>43528</v>
       </c>
-      <c r="PO1" s="63"/>
-      <c r="PP1" s="63"/>
-      <c r="PQ1" s="63"/>
-      <c r="PR1" s="63"/>
-      <c r="PS1" s="63"/>
-      <c r="PT1" s="63"/>
-      <c r="PU1" s="63">
+      <c r="PO1" s="39"/>
+      <c r="PP1" s="39"/>
+      <c r="PQ1" s="39"/>
+      <c r="PR1" s="39"/>
+      <c r="PS1" s="39"/>
+      <c r="PT1" s="39"/>
+      <c r="PU1" s="39">
         <v>43535</v>
       </c>
-      <c r="PV1" s="63"/>
-      <c r="PW1" s="63"/>
-      <c r="PX1" s="63"/>
-      <c r="PY1" s="63"/>
-      <c r="PZ1" s="63"/>
-      <c r="QA1" s="63"/>
-      <c r="QB1" s="63">
+      <c r="PV1" s="39"/>
+      <c r="PW1" s="39"/>
+      <c r="PX1" s="39"/>
+      <c r="PY1" s="39"/>
+      <c r="PZ1" s="39"/>
+      <c r="QA1" s="39"/>
+      <c r="QB1" s="39">
         <v>43542</v>
       </c>
-      <c r="QC1" s="63"/>
-      <c r="QD1" s="63"/>
-      <c r="QE1" s="63"/>
-      <c r="QF1" s="63"/>
-      <c r="QG1" s="63"/>
-      <c r="QH1" s="63"/>
-      <c r="QI1" s="63">
+      <c r="QC1" s="39"/>
+      <c r="QD1" s="39"/>
+      <c r="QE1" s="39"/>
+      <c r="QF1" s="39"/>
+      <c r="QG1" s="39"/>
+      <c r="QH1" s="39"/>
+      <c r="QI1" s="39">
         <v>43549</v>
       </c>
-      <c r="QJ1" s="63"/>
-      <c r="QK1" s="63"/>
-      <c r="QL1" s="63"/>
-      <c r="QM1" s="63"/>
-      <c r="QN1" s="63"/>
-      <c r="QO1" s="63"/>
-      <c r="QP1" s="63">
+      <c r="QJ1" s="39"/>
+      <c r="QK1" s="39"/>
+      <c r="QL1" s="39"/>
+      <c r="QM1" s="39"/>
+      <c r="QN1" s="39"/>
+      <c r="QO1" s="39"/>
+      <c r="QP1" s="39">
         <v>43556</v>
       </c>
-      <c r="QQ1" s="63"/>
-      <c r="QR1" s="63"/>
-      <c r="QS1" s="63"/>
-      <c r="QT1" s="63"/>
-      <c r="QU1" s="63"/>
-      <c r="QV1" s="63"/>
-      <c r="QW1" s="63">
+      <c r="QQ1" s="39"/>
+      <c r="QR1" s="39"/>
+      <c r="QS1" s="39"/>
+      <c r="QT1" s="39"/>
+      <c r="QU1" s="39"/>
+      <c r="QV1" s="39"/>
+      <c r="QW1" s="39">
         <v>43563</v>
       </c>
-      <c r="QX1" s="63"/>
-      <c r="QY1" s="63"/>
-      <c r="QZ1" s="63"/>
-      <c r="RA1" s="63"/>
-      <c r="RB1" s="63"/>
-      <c r="RC1" s="63"/>
-      <c r="RD1" s="63">
+      <c r="QX1" s="39"/>
+      <c r="QY1" s="39"/>
+      <c r="QZ1" s="39"/>
+      <c r="RA1" s="39"/>
+      <c r="RB1" s="39"/>
+      <c r="RC1" s="39"/>
+      <c r="RD1" s="39">
         <v>43570</v>
       </c>
-      <c r="RE1" s="63"/>
-      <c r="RF1" s="63"/>
-      <c r="RG1" s="63"/>
-      <c r="RH1" s="63"/>
-      <c r="RI1" s="63"/>
-      <c r="RJ1" s="63"/>
-      <c r="RK1" s="63">
+      <c r="RE1" s="39"/>
+      <c r="RF1" s="39"/>
+      <c r="RG1" s="39"/>
+      <c r="RH1" s="39"/>
+      <c r="RI1" s="39"/>
+      <c r="RJ1" s="39"/>
+      <c r="RK1" s="39">
         <v>43577</v>
       </c>
-      <c r="RL1" s="63"/>
-      <c r="RM1" s="63"/>
-      <c r="RN1" s="63"/>
-      <c r="RO1" s="63"/>
-      <c r="RP1" s="63"/>
-      <c r="RQ1" s="63"/>
-      <c r="RR1" s="63">
+      <c r="RL1" s="39"/>
+      <c r="RM1" s="39"/>
+      <c r="RN1" s="39"/>
+      <c r="RO1" s="39"/>
+      <c r="RP1" s="39"/>
+      <c r="RQ1" s="39"/>
+      <c r="RR1" s="39">
         <v>43584</v>
       </c>
-      <c r="RS1" s="63"/>
-      <c r="RT1" s="63"/>
-      <c r="RU1" s="63"/>
-      <c r="RV1" s="63"/>
-      <c r="RW1" s="63"/>
-      <c r="RX1" s="63"/>
-      <c r="RY1" s="63">
+      <c r="RS1" s="39"/>
+      <c r="RT1" s="39"/>
+      <c r="RU1" s="39"/>
+      <c r="RV1" s="39"/>
+      <c r="RW1" s="39"/>
+      <c r="RX1" s="39"/>
+      <c r="RY1" s="39">
         <v>43591</v>
       </c>
-      <c r="RZ1" s="63"/>
-      <c r="SA1" s="63"/>
-      <c r="SB1" s="63"/>
-      <c r="SC1" s="63"/>
-      <c r="SD1" s="63"/>
-      <c r="SE1" s="63"/>
-      <c r="SF1" s="63">
+      <c r="RZ1" s="39"/>
+      <c r="SA1" s="39"/>
+      <c r="SB1" s="39"/>
+      <c r="SC1" s="39"/>
+      <c r="SD1" s="39"/>
+      <c r="SE1" s="39"/>
+      <c r="SF1" s="39">
         <v>43598</v>
       </c>
-      <c r="SG1" s="63"/>
-      <c r="SH1" s="63"/>
-      <c r="SI1" s="63"/>
-      <c r="SJ1" s="63"/>
-      <c r="SK1" s="63"/>
-      <c r="SL1" s="63"/>
-      <c r="SM1" s="63">
+      <c r="SG1" s="39"/>
+      <c r="SH1" s="39"/>
+      <c r="SI1" s="39"/>
+      <c r="SJ1" s="39"/>
+      <c r="SK1" s="39"/>
+      <c r="SL1" s="39"/>
+      <c r="SM1" s="39">
         <v>43605</v>
       </c>
-      <c r="SN1" s="63"/>
-      <c r="SO1" s="63"/>
-      <c r="SP1" s="63"/>
-      <c r="SQ1" s="63"/>
-      <c r="SR1" s="63"/>
-      <c r="SS1" s="63"/>
-      <c r="ST1" s="63">
+      <c r="SN1" s="39"/>
+      <c r="SO1" s="39"/>
+      <c r="SP1" s="39"/>
+      <c r="SQ1" s="39"/>
+      <c r="SR1" s="39"/>
+      <c r="SS1" s="39"/>
+      <c r="ST1" s="39">
         <v>43612</v>
       </c>
-      <c r="SU1" s="63"/>
-      <c r="SV1" s="63"/>
-      <c r="SW1" s="63"/>
-      <c r="SX1" s="63"/>
-      <c r="SY1" s="63"/>
-      <c r="SZ1" s="63"/>
-      <c r="TA1" s="63">
+      <c r="SU1" s="39"/>
+      <c r="SV1" s="39"/>
+      <c r="SW1" s="39"/>
+      <c r="SX1" s="39"/>
+      <c r="SY1" s="39"/>
+      <c r="SZ1" s="39"/>
+      <c r="TA1" s="39">
         <v>43619</v>
       </c>
-      <c r="TB1" s="63"/>
-      <c r="TC1" s="63"/>
-      <c r="TD1" s="63"/>
-      <c r="TE1" s="63"/>
-      <c r="TF1" s="63"/>
-      <c r="TG1" s="63"/>
-      <c r="TH1" s="63">
+      <c r="TB1" s="39"/>
+      <c r="TC1" s="39"/>
+      <c r="TD1" s="39"/>
+      <c r="TE1" s="39"/>
+      <c r="TF1" s="39"/>
+      <c r="TG1" s="39"/>
+      <c r="TH1" s="39">
         <v>43626</v>
       </c>
-      <c r="TI1" s="63"/>
-      <c r="TJ1" s="63"/>
-      <c r="TK1" s="63"/>
-      <c r="TL1" s="63"/>
-      <c r="TM1" s="63"/>
-      <c r="TN1" s="63"/>
-      <c r="TO1" s="63">
+      <c r="TI1" s="39"/>
+      <c r="TJ1" s="39"/>
+      <c r="TK1" s="39"/>
+      <c r="TL1" s="39"/>
+      <c r="TM1" s="39"/>
+      <c r="TN1" s="39"/>
+      <c r="TO1" s="39">
         <v>43633</v>
       </c>
-      <c r="TP1" s="63"/>
-      <c r="TQ1" s="63"/>
-      <c r="TR1" s="63"/>
-      <c r="TS1" s="63"/>
-      <c r="TT1" s="63"/>
-      <c r="TU1" s="63"/>
-      <c r="TV1" s="63">
+      <c r="TP1" s="39"/>
+      <c r="TQ1" s="39"/>
+      <c r="TR1" s="39"/>
+      <c r="TS1" s="39"/>
+      <c r="TT1" s="39"/>
+      <c r="TU1" s="39"/>
+      <c r="TV1" s="39">
         <v>43640</v>
       </c>
-      <c r="TW1" s="63"/>
-      <c r="TX1" s="63"/>
-      <c r="TY1" s="63"/>
-      <c r="TZ1" s="63"/>
-      <c r="UA1" s="63"/>
-      <c r="UB1" s="63"/>
-      <c r="UC1" s="63">
+      <c r="TW1" s="39"/>
+      <c r="TX1" s="39"/>
+      <c r="TY1" s="39"/>
+      <c r="TZ1" s="39"/>
+      <c r="UA1" s="39"/>
+      <c r="UB1" s="39"/>
+      <c r="UC1" s="39">
         <v>43647</v>
       </c>
-      <c r="UD1" s="63"/>
-      <c r="UE1" s="63"/>
-      <c r="UF1" s="63"/>
-      <c r="UG1" s="63"/>
-      <c r="UH1" s="63"/>
-      <c r="UI1" s="63"/>
-      <c r="UJ1" s="63">
+      <c r="UD1" s="39"/>
+      <c r="UE1" s="39"/>
+      <c r="UF1" s="39"/>
+      <c r="UG1" s="39"/>
+      <c r="UH1" s="39"/>
+      <c r="UI1" s="39"/>
+      <c r="UJ1" s="39">
         <v>43654</v>
       </c>
-      <c r="UK1" s="63"/>
-      <c r="UL1" s="63"/>
-      <c r="UM1" s="63"/>
-      <c r="UN1" s="63"/>
-      <c r="UO1" s="63"/>
-      <c r="UP1" s="63"/>
-      <c r="UQ1" s="63">
+      <c r="UK1" s="39"/>
+      <c r="UL1" s="39"/>
+      <c r="UM1" s="39"/>
+      <c r="UN1" s="39"/>
+      <c r="UO1" s="39"/>
+      <c r="UP1" s="39"/>
+      <c r="UQ1" s="39">
         <v>43661</v>
       </c>
-      <c r="UR1" s="63"/>
-      <c r="US1" s="63"/>
-      <c r="UT1" s="63"/>
-      <c r="UU1" s="63"/>
-      <c r="UV1" s="63"/>
-      <c r="UW1" s="63"/>
-      <c r="UX1" s="63">
+      <c r="UR1" s="39"/>
+      <c r="US1" s="39"/>
+      <c r="UT1" s="39"/>
+      <c r="UU1" s="39"/>
+      <c r="UV1" s="39"/>
+      <c r="UW1" s="39"/>
+      <c r="UX1" s="39">
         <v>43668</v>
       </c>
-      <c r="UY1" s="63"/>
-      <c r="UZ1" s="63"/>
-      <c r="VA1" s="63"/>
-      <c r="VB1" s="63"/>
-      <c r="VC1" s="63"/>
-      <c r="VD1" s="63"/>
-      <c r="VE1" s="63">
+      <c r="UY1" s="39"/>
+      <c r="UZ1" s="39"/>
+      <c r="VA1" s="39"/>
+      <c r="VB1" s="39"/>
+      <c r="VC1" s="39"/>
+      <c r="VD1" s="39"/>
+      <c r="VE1" s="39">
         <v>43675</v>
       </c>
-      <c r="VF1" s="63"/>
-      <c r="VG1" s="63"/>
-      <c r="VH1" s="63"/>
-      <c r="VI1" s="63"/>
-      <c r="VJ1" s="63"/>
-      <c r="VK1" s="63"/>
-      <c r="VL1" s="63">
+      <c r="VF1" s="39"/>
+      <c r="VG1" s="39"/>
+      <c r="VH1" s="39"/>
+      <c r="VI1" s="39"/>
+      <c r="VJ1" s="39"/>
+      <c r="VK1" s="39"/>
+      <c r="VL1" s="39">
         <v>43682</v>
       </c>
-      <c r="VM1" s="63"/>
-      <c r="VN1" s="63"/>
-      <c r="VO1" s="63"/>
-      <c r="VP1" s="63"/>
-      <c r="VQ1" s="63"/>
-      <c r="VR1" s="63"/>
-      <c r="VS1" s="63">
+      <c r="VM1" s="39"/>
+      <c r="VN1" s="39"/>
+      <c r="VO1" s="39"/>
+      <c r="VP1" s="39"/>
+      <c r="VQ1" s="39"/>
+      <c r="VR1" s="39"/>
+      <c r="VS1" s="39">
         <v>43689</v>
       </c>
-      <c r="VT1" s="63"/>
-      <c r="VU1" s="63"/>
-      <c r="VV1" s="63"/>
-      <c r="VW1" s="63"/>
-      <c r="VX1" s="63"/>
-      <c r="VY1" s="63"/>
-      <c r="VZ1" s="63">
+      <c r="VT1" s="39"/>
+      <c r="VU1" s="39"/>
+      <c r="VV1" s="39"/>
+      <c r="VW1" s="39"/>
+      <c r="VX1" s="39"/>
+      <c r="VY1" s="39"/>
+      <c r="VZ1" s="39">
         <v>43696</v>
       </c>
-      <c r="WA1" s="63"/>
-      <c r="WB1" s="63"/>
-      <c r="WC1" s="63"/>
-      <c r="WD1" s="63"/>
-      <c r="WE1" s="63"/>
-      <c r="WF1" s="63"/>
-      <c r="WG1" s="63">
+      <c r="WA1" s="39"/>
+      <c r="WB1" s="39"/>
+      <c r="WC1" s="39"/>
+      <c r="WD1" s="39"/>
+      <c r="WE1" s="39"/>
+      <c r="WF1" s="39"/>
+      <c r="WG1" s="39">
         <v>43703</v>
       </c>
-      <c r="WH1" s="63"/>
-      <c r="WI1" s="63"/>
-      <c r="WJ1" s="63"/>
-      <c r="WK1" s="63"/>
-      <c r="WL1" s="63"/>
-      <c r="WM1" s="63"/>
-      <c r="WN1" s="63">
+      <c r="WH1" s="39"/>
+      <c r="WI1" s="39"/>
+      <c r="WJ1" s="39"/>
+      <c r="WK1" s="39"/>
+      <c r="WL1" s="39"/>
+      <c r="WM1" s="39"/>
+      <c r="WN1" s="39">
         <v>43710</v>
       </c>
-      <c r="WO1" s="63"/>
-      <c r="WP1" s="63"/>
-      <c r="WQ1" s="63"/>
-      <c r="WR1" s="63"/>
-      <c r="WS1" s="63"/>
-      <c r="WT1" s="63"/>
-      <c r="WU1" s="63">
+      <c r="WO1" s="39"/>
+      <c r="WP1" s="39"/>
+      <c r="WQ1" s="39"/>
+      <c r="WR1" s="39"/>
+      <c r="WS1" s="39"/>
+      <c r="WT1" s="39"/>
+      <c r="WU1" s="39">
         <v>43717</v>
       </c>
-      <c r="WV1" s="63"/>
-      <c r="WW1" s="63"/>
-      <c r="WX1" s="63"/>
-      <c r="WY1" s="63"/>
-      <c r="WZ1" s="63"/>
-      <c r="XA1" s="63"/>
-      <c r="XB1" s="63">
+      <c r="WV1" s="39"/>
+      <c r="WW1" s="39"/>
+      <c r="WX1" s="39"/>
+      <c r="WY1" s="39"/>
+      <c r="WZ1" s="39"/>
+      <c r="XA1" s="39"/>
+      <c r="XB1" s="39">
         <v>43724</v>
       </c>
-      <c r="XC1" s="63"/>
-      <c r="XD1" s="63"/>
-      <c r="XE1" s="63"/>
-      <c r="XF1" s="63"/>
-      <c r="XG1" s="63"/>
-      <c r="XH1" s="63"/>
-      <c r="XI1" s="63">
+      <c r="XC1" s="39"/>
+      <c r="XD1" s="39"/>
+      <c r="XE1" s="39"/>
+      <c r="XF1" s="39"/>
+      <c r="XG1" s="39"/>
+      <c r="XH1" s="39"/>
+      <c r="XI1" s="39">
         <v>43731</v>
       </c>
-      <c r="XJ1" s="63"/>
-      <c r="XK1" s="63"/>
-      <c r="XL1" s="63"/>
-      <c r="XM1" s="63"/>
-      <c r="XN1" s="63"/>
-      <c r="XO1" s="63"/>
-      <c r="XP1" s="63">
+      <c r="XJ1" s="39"/>
+      <c r="XK1" s="39"/>
+      <c r="XL1" s="39"/>
+      <c r="XM1" s="39"/>
+      <c r="XN1" s="39"/>
+      <c r="XO1" s="39"/>
+      <c r="XP1" s="39">
         <v>43738</v>
       </c>
-      <c r="XQ1" s="63"/>
-      <c r="XR1" s="63"/>
-      <c r="XS1" s="63"/>
-      <c r="XT1" s="63"/>
-      <c r="XU1" s="63"/>
-      <c r="XV1" s="63"/>
-      <c r="XW1" s="63">
+      <c r="XQ1" s="39"/>
+      <c r="XR1" s="39"/>
+      <c r="XS1" s="39"/>
+      <c r="XT1" s="39"/>
+      <c r="XU1" s="39"/>
+      <c r="XV1" s="39"/>
+      <c r="XW1" s="39">
         <v>43745</v>
       </c>
-      <c r="XX1" s="63"/>
-      <c r="XY1" s="63"/>
-      <c r="XZ1" s="63"/>
-      <c r="YA1" s="63"/>
-      <c r="YB1" s="63"/>
-      <c r="YC1" s="63"/>
-      <c r="YD1" s="63">
+      <c r="XX1" s="39"/>
+      <c r="XY1" s="39"/>
+      <c r="XZ1" s="39"/>
+      <c r="YA1" s="39"/>
+      <c r="YB1" s="39"/>
+      <c r="YC1" s="39"/>
+      <c r="YD1" s="39">
         <v>43752</v>
       </c>
-      <c r="YE1" s="63"/>
-      <c r="YF1" s="63"/>
-      <c r="YG1" s="63"/>
-      <c r="YH1" s="63"/>
-      <c r="YI1" s="63"/>
-      <c r="YJ1" s="63"/>
-      <c r="YK1" s="63">
+      <c r="YE1" s="39"/>
+      <c r="YF1" s="39"/>
+      <c r="YG1" s="39"/>
+      <c r="YH1" s="39"/>
+      <c r="YI1" s="39"/>
+      <c r="YJ1" s="39"/>
+      <c r="YK1" s="39">
         <v>43759</v>
       </c>
-      <c r="YL1" s="63"/>
-      <c r="YM1" s="63"/>
-      <c r="YN1" s="63"/>
-      <c r="YO1" s="63"/>
-      <c r="YP1" s="63"/>
-      <c r="YQ1" s="63"/>
-      <c r="YR1" s="63">
+      <c r="YL1" s="39"/>
+      <c r="YM1" s="39"/>
+      <c r="YN1" s="39"/>
+      <c r="YO1" s="39"/>
+      <c r="YP1" s="39"/>
+      <c r="YQ1" s="39"/>
+      <c r="YR1" s="39">
         <v>43766</v>
       </c>
-      <c r="YS1" s="63"/>
-      <c r="YT1" s="63"/>
-      <c r="YU1" s="63"/>
-      <c r="YV1" s="63"/>
-      <c r="YW1" s="63"/>
-      <c r="YX1" s="63"/>
-      <c r="YY1" s="63">
+      <c r="YS1" s="39"/>
+      <c r="YT1" s="39"/>
+      <c r="YU1" s="39"/>
+      <c r="YV1" s="39"/>
+      <c r="YW1" s="39"/>
+      <c r="YX1" s="39"/>
+      <c r="YY1" s="39">
         <v>43773</v>
       </c>
-      <c r="YZ1" s="63"/>
-      <c r="ZA1" s="63"/>
-      <c r="ZB1" s="63"/>
-      <c r="ZC1" s="63"/>
-      <c r="ZD1" s="63"/>
-      <c r="ZE1" s="63"/>
-      <c r="ZF1" s="63">
+      <c r="YZ1" s="39"/>
+      <c r="ZA1" s="39"/>
+      <c r="ZB1" s="39"/>
+      <c r="ZC1" s="39"/>
+      <c r="ZD1" s="39"/>
+      <c r="ZE1" s="39"/>
+      <c r="ZF1" s="39">
         <v>43780</v>
       </c>
-      <c r="ZG1" s="63"/>
-      <c r="ZH1" s="63"/>
-      <c r="ZI1" s="63"/>
-      <c r="ZJ1" s="63"/>
-      <c r="ZK1" s="63"/>
-      <c r="ZL1" s="63"/>
-      <c r="ZM1" s="63">
+      <c r="ZG1" s="39"/>
+      <c r="ZH1" s="39"/>
+      <c r="ZI1" s="39"/>
+      <c r="ZJ1" s="39"/>
+      <c r="ZK1" s="39"/>
+      <c r="ZL1" s="39"/>
+      <c r="ZM1" s="39">
         <v>43787</v>
       </c>
-      <c r="ZN1" s="63"/>
-      <c r="ZO1" s="63"/>
-      <c r="ZP1" s="63"/>
-      <c r="ZQ1" s="63"/>
-      <c r="ZR1" s="63"/>
-      <c r="ZS1" s="63"/>
-      <c r="ZT1" s="63">
+      <c r="ZN1" s="39"/>
+      <c r="ZO1" s="39"/>
+      <c r="ZP1" s="39"/>
+      <c r="ZQ1" s="39"/>
+      <c r="ZR1" s="39"/>
+      <c r="ZS1" s="39"/>
+      <c r="ZT1" s="39">
         <v>43794</v>
       </c>
-      <c r="ZU1" s="63"/>
-      <c r="ZV1" s="63"/>
-      <c r="ZW1" s="63"/>
-      <c r="ZX1" s="63"/>
-      <c r="ZY1" s="63"/>
-      <c r="ZZ1" s="63"/>
-      <c r="AAA1" s="63">
+      <c r="ZU1" s="39"/>
+      <c r="ZV1" s="39"/>
+      <c r="ZW1" s="39"/>
+      <c r="ZX1" s="39"/>
+      <c r="ZY1" s="39"/>
+      <c r="ZZ1" s="39"/>
+      <c r="AAA1" s="39">
         <v>43801</v>
       </c>
-      <c r="AAB1" s="63"/>
-      <c r="AAC1" s="63"/>
-      <c r="AAD1" s="63"/>
-      <c r="AAE1" s="63"/>
-      <c r="AAF1" s="63"/>
-      <c r="AAG1" s="63"/>
-      <c r="AAH1" s="63">
+      <c r="AAB1" s="39"/>
+      <c r="AAC1" s="39"/>
+      <c r="AAD1" s="39"/>
+      <c r="AAE1" s="39"/>
+      <c r="AAF1" s="39"/>
+      <c r="AAG1" s="39"/>
+      <c r="AAH1" s="39">
         <v>43808</v>
       </c>
-      <c r="AAI1" s="63"/>
-      <c r="AAJ1" s="63"/>
-      <c r="AAK1" s="63"/>
-      <c r="AAL1" s="63"/>
-      <c r="AAM1" s="63"/>
-      <c r="AAN1" s="63"/>
-      <c r="AAO1" s="63">
+      <c r="AAI1" s="39"/>
+      <c r="AAJ1" s="39"/>
+      <c r="AAK1" s="39"/>
+      <c r="AAL1" s="39"/>
+      <c r="AAM1" s="39"/>
+      <c r="AAN1" s="39"/>
+      <c r="AAO1" s="39">
         <v>43815</v>
       </c>
-      <c r="AAP1" s="63"/>
-      <c r="AAQ1" s="63"/>
-      <c r="AAR1" s="63"/>
-      <c r="AAS1" s="63"/>
-      <c r="AAT1" s="63"/>
-      <c r="AAU1" s="63"/>
-      <c r="AAV1" s="63">
+      <c r="AAP1" s="39"/>
+      <c r="AAQ1" s="39"/>
+      <c r="AAR1" s="39"/>
+      <c r="AAS1" s="39"/>
+      <c r="AAT1" s="39"/>
+      <c r="AAU1" s="39"/>
+      <c r="AAV1" s="39">
         <v>43822</v>
       </c>
-      <c r="AAW1" s="63"/>
-      <c r="AAX1" s="63"/>
-      <c r="AAY1" s="63"/>
-      <c r="AAZ1" s="63"/>
-      <c r="ABA1" s="63"/>
-      <c r="ABB1" s="63"/>
-      <c r="ABC1" s="63">
+      <c r="AAW1" s="39"/>
+      <c r="AAX1" s="39"/>
+      <c r="AAY1" s="39"/>
+      <c r="AAZ1" s="39"/>
+      <c r="ABA1" s="39"/>
+      <c r="ABB1" s="39"/>
+      <c r="ABC1" s="39">
         <v>43829</v>
       </c>
-      <c r="ABD1" s="63"/>
-      <c r="ABE1" s="63"/>
-      <c r="ABF1" s="63"/>
-      <c r="ABG1" s="63"/>
-      <c r="ABH1" s="63"/>
-      <c r="ABI1" s="63"/>
+      <c r="ABD1" s="39"/>
+      <c r="ABE1" s="39"/>
+      <c r="ABF1" s="39"/>
+      <c r="ABG1" s="39"/>
+      <c r="ABH1" s="39"/>
+      <c r="ABI1" s="39"/>
     </row>
     <row r="2" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -7260,415 +7282,415 @@
       <c r="B2" t="s">
         <v>139</v>
       </c>
-      <c r="GS2" s="38" t="s">
+      <c r="GS2" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="GT2" s="38"/>
-      <c r="GU2" s="38"/>
-      <c r="GV2" s="38"/>
-      <c r="GW2" s="38"/>
-      <c r="GX2" s="38"/>
-      <c r="GY2" s="38"/>
-      <c r="GZ2" s="38"/>
-      <c r="HA2" s="38"/>
-      <c r="HB2" s="38"/>
-      <c r="HC2" s="38"/>
-      <c r="HD2" s="38"/>
-      <c r="HE2" s="38"/>
-      <c r="HF2" s="38"/>
-      <c r="HG2" s="38"/>
-      <c r="HH2" s="38"/>
-      <c r="HI2" s="38"/>
-      <c r="HJ2" s="38"/>
-      <c r="HK2" s="38"/>
-      <c r="HL2" s="38"/>
-      <c r="HM2" s="38"/>
-      <c r="HN2" s="40" t="s">
+      <c r="GT2" s="44"/>
+      <c r="GU2" s="44"/>
+      <c r="GV2" s="44"/>
+      <c r="GW2" s="44"/>
+      <c r="GX2" s="44"/>
+      <c r="GY2" s="44"/>
+      <c r="GZ2" s="44"/>
+      <c r="HA2" s="44"/>
+      <c r="HB2" s="44"/>
+      <c r="HC2" s="44"/>
+      <c r="HD2" s="44"/>
+      <c r="HE2" s="44"/>
+      <c r="HF2" s="44"/>
+      <c r="HG2" s="44"/>
+      <c r="HH2" s="44"/>
+      <c r="HI2" s="44"/>
+      <c r="HJ2" s="44"/>
+      <c r="HK2" s="44"/>
+      <c r="HL2" s="44"/>
+      <c r="HM2" s="44"/>
+      <c r="HN2" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="HO2" s="40"/>
-      <c r="HP2" s="40"/>
-      <c r="HQ2" s="40"/>
-      <c r="HR2" s="40"/>
-      <c r="HS2" s="40"/>
-      <c r="HT2" s="40"/>
-      <c r="HU2" s="41" t="s">
+      <c r="HO2" s="45"/>
+      <c r="HP2" s="45"/>
+      <c r="HQ2" s="45"/>
+      <c r="HR2" s="45"/>
+      <c r="HS2" s="45"/>
+      <c r="HT2" s="45"/>
+      <c r="HU2" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="HV2" s="40" t="s">
+      <c r="HV2" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="HW2" s="40"/>
-      <c r="HX2" s="40"/>
-      <c r="HY2" s="40"/>
-      <c r="HZ2" s="40"/>
-      <c r="IA2" s="40"/>
-      <c r="IB2" s="40"/>
-      <c r="IC2" s="42" t="s">
+      <c r="HW2" s="45"/>
+      <c r="HX2" s="45"/>
+      <c r="HY2" s="45"/>
+      <c r="HZ2" s="45"/>
+      <c r="IA2" s="45"/>
+      <c r="IB2" s="45"/>
+      <c r="IC2" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="ID2" s="42"/>
-      <c r="IE2" s="42"/>
-      <c r="IF2" s="42"/>
-      <c r="IG2" s="42"/>
-      <c r="IH2" s="42"/>
-      <c r="II2" s="42"/>
-      <c r="IJ2" s="43" t="s">
+      <c r="ID2" s="46"/>
+      <c r="IE2" s="46"/>
+      <c r="IF2" s="46"/>
+      <c r="IG2" s="46"/>
+      <c r="IH2" s="46"/>
+      <c r="II2" s="46"/>
+      <c r="IJ2" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="IK2" s="44" t="s">
+      <c r="IK2" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="IL2" s="44"/>
-      <c r="IM2" s="44"/>
-      <c r="IN2" s="44"/>
-      <c r="IO2" s="44"/>
-      <c r="IP2" s="44"/>
-      <c r="IQ2" s="44"/>
-      <c r="IR2" s="44"/>
-      <c r="IS2" s="44"/>
-      <c r="IT2" s="44"/>
-      <c r="IU2" s="44"/>
-      <c r="IV2" s="44" t="s">
+      <c r="IL2" s="40"/>
+      <c r="IM2" s="40"/>
+      <c r="IN2" s="40"/>
+      <c r="IO2" s="40"/>
+      <c r="IP2" s="40"/>
+      <c r="IQ2" s="40"/>
+      <c r="IR2" s="40"/>
+      <c r="IS2" s="40"/>
+      <c r="IT2" s="40"/>
+      <c r="IU2" s="40"/>
+      <c r="IV2" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="IW2" s="44"/>
-      <c r="IX2" s="44"/>
-      <c r="IY2" s="44" t="s">
+      <c r="IW2" s="40"/>
+      <c r="IX2" s="40"/>
+      <c r="IY2" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="IZ2" s="44"/>
-      <c r="JA2" s="44"/>
-      <c r="JB2" s="44"/>
-      <c r="JC2" s="45" t="s">
+      <c r="IZ2" s="40"/>
+      <c r="JA2" s="40"/>
+      <c r="JB2" s="40"/>
+      <c r="JC2" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="JD2" s="45"/>
-      <c r="JE2" s="45"/>
-      <c r="JF2" s="45"/>
-      <c r="JG2" s="45"/>
-      <c r="JH2" s="45"/>
-      <c r="JI2" s="45"/>
-      <c r="JJ2" s="45"/>
-      <c r="JK2" s="45"/>
-      <c r="JL2" s="45" t="s">
+      <c r="JD2" s="41"/>
+      <c r="JE2" s="41"/>
+      <c r="JF2" s="41"/>
+      <c r="JG2" s="41"/>
+      <c r="JH2" s="41"/>
+      <c r="JI2" s="41"/>
+      <c r="JJ2" s="41"/>
+      <c r="JK2" s="41"/>
+      <c r="JL2" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="JM2" s="45"/>
-      <c r="JN2" s="45"/>
-      <c r="JO2" s="45"/>
-      <c r="JP2" s="45"/>
-      <c r="JQ2" s="45"/>
-      <c r="JR2" s="45"/>
-      <c r="JS2" s="45"/>
-      <c r="JT2" s="45"/>
-      <c r="JU2" s="45"/>
-      <c r="JV2" s="45"/>
-      <c r="JW2" s="45"/>
-      <c r="JX2" s="45"/>
-      <c r="JY2" s="45"/>
-      <c r="JZ2" s="45"/>
-      <c r="KA2" s="45"/>
-      <c r="KB2" s="45"/>
-      <c r="KC2" s="45"/>
-      <c r="KD2" s="45"/>
-      <c r="KE2" s="45"/>
-      <c r="KF2" s="45"/>
-      <c r="KG2" s="45"/>
-      <c r="KH2" s="45"/>
-      <c r="KI2" s="45"/>
-      <c r="KJ2" s="45"/>
-      <c r="KK2" s="45"/>
-      <c r="KL2" s="46" t="s">
+      <c r="JM2" s="41"/>
+      <c r="JN2" s="41"/>
+      <c r="JO2" s="41"/>
+      <c r="JP2" s="41"/>
+      <c r="JQ2" s="41"/>
+      <c r="JR2" s="41"/>
+      <c r="JS2" s="41"/>
+      <c r="JT2" s="41"/>
+      <c r="JU2" s="41"/>
+      <c r="JV2" s="41"/>
+      <c r="JW2" s="41"/>
+      <c r="JX2" s="41"/>
+      <c r="JY2" s="41"/>
+      <c r="JZ2" s="41"/>
+      <c r="KA2" s="41"/>
+      <c r="KB2" s="41"/>
+      <c r="KC2" s="41"/>
+      <c r="KD2" s="41"/>
+      <c r="KE2" s="41"/>
+      <c r="KF2" s="41"/>
+      <c r="KG2" s="41"/>
+      <c r="KH2" s="41"/>
+      <c r="KI2" s="41"/>
+      <c r="KJ2" s="41"/>
+      <c r="KK2" s="41"/>
+      <c r="KL2" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="KM2" s="46"/>
-      <c r="KN2" s="46"/>
-      <c r="KO2" s="46"/>
-      <c r="KP2" s="46"/>
-      <c r="KQ2" s="46"/>
-      <c r="KR2" s="46"/>
-      <c r="KS2" s="46"/>
-      <c r="KT2" s="46"/>
-      <c r="KU2" s="47" t="s">
+      <c r="KM2" s="42"/>
+      <c r="KN2" s="42"/>
+      <c r="KO2" s="42"/>
+      <c r="KP2" s="42"/>
+      <c r="KQ2" s="42"/>
+      <c r="KR2" s="42"/>
+      <c r="KS2" s="42"/>
+      <c r="KT2" s="42"/>
+      <c r="KU2" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="KV2" s="47"/>
-      <c r="KW2" s="47"/>
-      <c r="KX2" s="47"/>
-      <c r="KY2" s="47"/>
-      <c r="KZ2" s="47"/>
-      <c r="LA2" s="47"/>
-      <c r="LB2" s="47"/>
-      <c r="LC2" s="47"/>
-      <c r="LD2" s="47"/>
-      <c r="LE2" s="47"/>
-      <c r="LF2" s="47"/>
-      <c r="LG2" s="47"/>
-      <c r="LH2" s="47"/>
-      <c r="LI2" s="47"/>
-      <c r="LJ2" s="47"/>
-      <c r="LK2" s="47"/>
-      <c r="LL2" s="47"/>
-      <c r="LM2" s="47"/>
-      <c r="LN2" s="47"/>
-      <c r="LO2" s="44" t="s">
+      <c r="KV2" s="43"/>
+      <c r="KW2" s="43"/>
+      <c r="KX2" s="43"/>
+      <c r="KY2" s="43"/>
+      <c r="KZ2" s="43"/>
+      <c r="LA2" s="43"/>
+      <c r="LB2" s="43"/>
+      <c r="LC2" s="43"/>
+      <c r="LD2" s="43"/>
+      <c r="LE2" s="43"/>
+      <c r="LF2" s="43"/>
+      <c r="LG2" s="43"/>
+      <c r="LH2" s="43"/>
+      <c r="LI2" s="43"/>
+      <c r="LJ2" s="43"/>
+      <c r="LK2" s="43"/>
+      <c r="LL2" s="43"/>
+      <c r="LM2" s="43"/>
+      <c r="LN2" s="43"/>
+      <c r="LO2" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="LP2" s="44"/>
-      <c r="LQ2" s="44"/>
-      <c r="LR2" s="44"/>
-      <c r="LS2" s="44"/>
-      <c r="LT2" s="44"/>
-      <c r="LU2" s="44"/>
-      <c r="LV2" s="44"/>
-      <c r="LW2" s="44"/>
-      <c r="NG2" s="49" t="s">
+      <c r="LP2" s="40"/>
+      <c r="LQ2" s="40"/>
+      <c r="LR2" s="40"/>
+      <c r="LS2" s="40"/>
+      <c r="LT2" s="40"/>
+      <c r="LU2" s="40"/>
+      <c r="LV2" s="40"/>
+      <c r="LW2" s="40"/>
+      <c r="NG2" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="NH2" s="49"/>
-      <c r="NI2" s="49"/>
-      <c r="NJ2" s="49"/>
-      <c r="NK2" s="49"/>
-      <c r="NL2" s="49"/>
-      <c r="NM2" s="49"/>
-      <c r="NN2" s="49"/>
-      <c r="NO2" s="49"/>
-      <c r="NP2" s="49"/>
-      <c r="NQ2" s="49"/>
-      <c r="NR2" s="49"/>
-      <c r="NS2" s="49"/>
-      <c r="NT2" s="49"/>
-      <c r="NU2" s="49"/>
-      <c r="NV2" s="49"/>
-      <c r="NW2" s="49"/>
-      <c r="NX2" s="49"/>
-      <c r="NY2" s="49"/>
-      <c r="NZ2" s="49"/>
-      <c r="OA2" s="49"/>
-      <c r="OB2" s="49"/>
-      <c r="OO2" s="57" t="s">
+      <c r="NH2" s="50"/>
+      <c r="NI2" s="50"/>
+      <c r="NJ2" s="50"/>
+      <c r="NK2" s="50"/>
+      <c r="NL2" s="50"/>
+      <c r="NM2" s="50"/>
+      <c r="NN2" s="50"/>
+      <c r="NO2" s="50"/>
+      <c r="NP2" s="50"/>
+      <c r="NQ2" s="50"/>
+      <c r="NR2" s="50"/>
+      <c r="NS2" s="50"/>
+      <c r="NT2" s="50"/>
+      <c r="NU2" s="50"/>
+      <c r="NV2" s="50"/>
+      <c r="NW2" s="50"/>
+      <c r="NX2" s="50"/>
+      <c r="NY2" s="50"/>
+      <c r="NZ2" s="50"/>
+      <c r="OA2" s="50"/>
+      <c r="OB2" s="50"/>
+      <c r="OO2" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="OP2" s="58"/>
-      <c r="OQ2" s="58"/>
-      <c r="OR2" s="58"/>
-      <c r="OS2" s="45"/>
-      <c r="OT2" s="45"/>
-      <c r="OU2" s="45"/>
-      <c r="OV2" s="45"/>
-      <c r="OW2" s="45"/>
-      <c r="OX2" s="45"/>
-      <c r="OY2" s="45"/>
-      <c r="OZ2" s="45"/>
-      <c r="PA2" s="45"/>
-      <c r="PB2" s="45"/>
-      <c r="PC2" s="45"/>
-      <c r="PD2" s="45"/>
-      <c r="PE2" s="45"/>
-      <c r="PF2" s="45"/>
-      <c r="PG2" s="45"/>
-      <c r="PH2" s="45"/>
-      <c r="PI2" s="45"/>
-      <c r="PJ2" s="45"/>
-      <c r="PK2" s="45"/>
-      <c r="PL2" s="45"/>
-      <c r="PM2" s="45"/>
-      <c r="PN2" s="45"/>
-      <c r="PO2" s="45"/>
-      <c r="PP2" s="45"/>
-      <c r="PQ2" s="45"/>
-      <c r="PR2" s="45"/>
-      <c r="PS2" s="45"/>
-      <c r="PT2" s="45"/>
-      <c r="PU2" s="45"/>
-      <c r="PV2" s="45"/>
-      <c r="PW2" s="45"/>
-      <c r="PX2" s="45"/>
-      <c r="PY2" s="45"/>
-      <c r="PZ2" s="45"/>
-      <c r="QA2" s="45"/>
-      <c r="QB2" s="45"/>
-      <c r="QC2" s="45"/>
-      <c r="QD2" s="45"/>
-      <c r="QE2" s="45"/>
-      <c r="QF2" s="45"/>
-      <c r="QG2" s="45"/>
-      <c r="QH2" s="45"/>
-      <c r="QI2" s="45"/>
-      <c r="QJ2" s="45"/>
-      <c r="QK2" s="45"/>
-      <c r="QL2" s="45"/>
-      <c r="QM2" s="45"/>
-      <c r="QN2" s="45"/>
-      <c r="QO2" s="45"/>
-      <c r="QP2" s="45"/>
-      <c r="QQ2" s="40" t="s">
+      <c r="OP2" s="49"/>
+      <c r="OQ2" s="49"/>
+      <c r="OR2" s="49"/>
+      <c r="OS2" s="41"/>
+      <c r="OT2" s="41"/>
+      <c r="OU2" s="41"/>
+      <c r="OV2" s="41"/>
+      <c r="OW2" s="41"/>
+      <c r="OX2" s="41"/>
+      <c r="OY2" s="41"/>
+      <c r="OZ2" s="41"/>
+      <c r="PA2" s="41"/>
+      <c r="PB2" s="41"/>
+      <c r="PC2" s="41"/>
+      <c r="PD2" s="41"/>
+      <c r="PE2" s="41"/>
+      <c r="PF2" s="41"/>
+      <c r="PG2" s="41"/>
+      <c r="PH2" s="41"/>
+      <c r="PI2" s="41"/>
+      <c r="PJ2" s="41"/>
+      <c r="PK2" s="41"/>
+      <c r="PL2" s="41"/>
+      <c r="PM2" s="41"/>
+      <c r="PN2" s="41"/>
+      <c r="PO2" s="41"/>
+      <c r="PP2" s="41"/>
+      <c r="PQ2" s="41"/>
+      <c r="PR2" s="41"/>
+      <c r="PS2" s="41"/>
+      <c r="PT2" s="41"/>
+      <c r="PU2" s="41"/>
+      <c r="PV2" s="41"/>
+      <c r="PW2" s="41"/>
+      <c r="PX2" s="41"/>
+      <c r="PY2" s="41"/>
+      <c r="PZ2" s="41"/>
+      <c r="QA2" s="41"/>
+      <c r="QB2" s="41"/>
+      <c r="QC2" s="41"/>
+      <c r="QD2" s="41"/>
+      <c r="QE2" s="41"/>
+      <c r="QF2" s="41"/>
+      <c r="QG2" s="41"/>
+      <c r="QH2" s="41"/>
+      <c r="QI2" s="41"/>
+      <c r="QJ2" s="41"/>
+      <c r="QK2" s="41"/>
+      <c r="QL2" s="41"/>
+      <c r="QM2" s="41"/>
+      <c r="QN2" s="41"/>
+      <c r="QO2" s="41"/>
+      <c r="QP2" s="41"/>
+      <c r="QQ2" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="QR2" s="40"/>
-      <c r="QS2" s="40"/>
-      <c r="QT2" s="40"/>
-      <c r="QU2" s="40"/>
-      <c r="QV2" s="40"/>
-      <c r="QW2" s="40"/>
-      <c r="QX2" s="47" t="s">
+      <c r="QR2" s="45"/>
+      <c r="QS2" s="45"/>
+      <c r="QT2" s="45"/>
+      <c r="QU2" s="45"/>
+      <c r="QV2" s="45"/>
+      <c r="QW2" s="45"/>
+      <c r="QX2" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="QY2" s="47"/>
-      <c r="QZ2" s="47"/>
-      <c r="RA2" s="47"/>
-      <c r="RB2" s="47"/>
-      <c r="RC2" s="47"/>
-      <c r="RD2" s="47"/>
-      <c r="RE2" s="47"/>
-      <c r="RF2" s="47"/>
-      <c r="RG2" s="47"/>
-      <c r="RH2" s="47"/>
-      <c r="RI2" s="47"/>
-      <c r="RJ2" s="47"/>
-      <c r="RK2" s="47"/>
-      <c r="RL2" s="47"/>
-      <c r="RM2" s="47"/>
-      <c r="RN2" s="47"/>
-      <c r="RO2" s="40" t="s">
+      <c r="QY2" s="43"/>
+      <c r="QZ2" s="43"/>
+      <c r="RA2" s="43"/>
+      <c r="RB2" s="43"/>
+      <c r="RC2" s="43"/>
+      <c r="RD2" s="43"/>
+      <c r="RE2" s="43"/>
+      <c r="RF2" s="43"/>
+      <c r="RG2" s="43"/>
+      <c r="RH2" s="43"/>
+      <c r="RI2" s="43"/>
+      <c r="RJ2" s="43"/>
+      <c r="RK2" s="43"/>
+      <c r="RL2" s="43"/>
+      <c r="RM2" s="43"/>
+      <c r="RN2" s="43"/>
+      <c r="RO2" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="RP2" s="40"/>
-      <c r="RQ2" s="40"/>
-      <c r="RR2" s="40"/>
-      <c r="RS2" s="40"/>
-      <c r="RT2" s="40"/>
-      <c r="RU2" s="40"/>
-      <c r="RV2" s="38" t="s">
+      <c r="RP2" s="45"/>
+      <c r="RQ2" s="45"/>
+      <c r="RR2" s="45"/>
+      <c r="RS2" s="45"/>
+      <c r="RT2" s="45"/>
+      <c r="RU2" s="45"/>
+      <c r="RV2" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="RW2" s="38"/>
-      <c r="RX2" s="38"/>
-      <c r="RY2" s="38"/>
-      <c r="RZ2" s="38"/>
-      <c r="SA2" s="42" t="s">
+      <c r="RW2" s="44"/>
+      <c r="RX2" s="44"/>
+      <c r="RY2" s="44"/>
+      <c r="RZ2" s="44"/>
+      <c r="SA2" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="SB2" s="42"/>
-      <c r="SC2" s="42"/>
-      <c r="SD2" s="42"/>
-      <c r="SE2" s="42"/>
-      <c r="SF2" s="42"/>
-      <c r="SG2" s="42"/>
-      <c r="SH2" s="42"/>
-      <c r="SI2" s="42"/>
-      <c r="SJ2" s="42"/>
-      <c r="SK2" s="42"/>
-      <c r="SL2" s="42"/>
-      <c r="SM2" s="42"/>
-      <c r="SN2" s="42"/>
-      <c r="SO2" s="42"/>
-      <c r="SP2" s="42"/>
-      <c r="SQ2" s="42"/>
-      <c r="SR2" s="42"/>
-      <c r="SS2" s="42"/>
-      <c r="ST2" s="42"/>
-      <c r="SU2" s="42"/>
-      <c r="SV2" s="42"/>
-      <c r="SW2" s="42"/>
-      <c r="SX2" s="42"/>
-      <c r="SY2" s="42"/>
-      <c r="SZ2" s="42"/>
-      <c r="TA2" s="42"/>
-      <c r="TB2" s="42"/>
-      <c r="TC2" s="42"/>
-      <c r="TD2" s="42"/>
-      <c r="TE2" s="42"/>
-      <c r="TF2" s="42"/>
-      <c r="TG2" s="42"/>
-      <c r="TH2" s="42"/>
-      <c r="TI2" s="42"/>
-      <c r="TJ2" s="42"/>
-      <c r="TK2" s="42"/>
-      <c r="TL2" s="42"/>
-      <c r="TM2" s="42"/>
-      <c r="TN2" s="42"/>
-      <c r="TO2" s="42"/>
-      <c r="TP2" s="42"/>
-      <c r="TQ2" s="42"/>
-      <c r="TR2" s="42"/>
-      <c r="TS2" s="42"/>
-      <c r="TT2" s="42"/>
-      <c r="TU2" s="42"/>
-      <c r="TV2" s="42"/>
-      <c r="TW2" s="42"/>
-      <c r="TX2" s="50" t="s">
+      <c r="SB2" s="46"/>
+      <c r="SC2" s="46"/>
+      <c r="SD2" s="46"/>
+      <c r="SE2" s="46"/>
+      <c r="SF2" s="46"/>
+      <c r="SG2" s="46"/>
+      <c r="SH2" s="46"/>
+      <c r="SI2" s="46"/>
+      <c r="SJ2" s="46"/>
+      <c r="SK2" s="46"/>
+      <c r="SL2" s="46"/>
+      <c r="SM2" s="46"/>
+      <c r="SN2" s="46"/>
+      <c r="SO2" s="46"/>
+      <c r="SP2" s="46"/>
+      <c r="SQ2" s="46"/>
+      <c r="SR2" s="46"/>
+      <c r="SS2" s="46"/>
+      <c r="ST2" s="46"/>
+      <c r="SU2" s="46"/>
+      <c r="SV2" s="46"/>
+      <c r="SW2" s="46"/>
+      <c r="SX2" s="46"/>
+      <c r="SY2" s="46"/>
+      <c r="SZ2" s="46"/>
+      <c r="TA2" s="46"/>
+      <c r="TB2" s="46"/>
+      <c r="TC2" s="46"/>
+      <c r="TD2" s="46"/>
+      <c r="TE2" s="46"/>
+      <c r="TF2" s="46"/>
+      <c r="TG2" s="46"/>
+      <c r="TH2" s="46"/>
+      <c r="TI2" s="46"/>
+      <c r="TJ2" s="46"/>
+      <c r="TK2" s="46"/>
+      <c r="TL2" s="46"/>
+      <c r="TM2" s="46"/>
+      <c r="TN2" s="46"/>
+      <c r="TO2" s="46"/>
+      <c r="TP2" s="46"/>
+      <c r="TQ2" s="46"/>
+      <c r="TR2" s="46"/>
+      <c r="TS2" s="46"/>
+      <c r="TT2" s="46"/>
+      <c r="TU2" s="46"/>
+      <c r="TV2" s="46"/>
+      <c r="TW2" s="46"/>
+      <c r="TX2" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="TY2" s="50"/>
-      <c r="TZ2" s="50"/>
-      <c r="UA2" s="50"/>
-      <c r="UB2" s="50"/>
-      <c r="UC2" s="50"/>
-      <c r="UD2" s="50"/>
-      <c r="UE2" s="50"/>
-      <c r="UF2" s="50"/>
-      <c r="UG2" s="50"/>
-      <c r="UH2" s="50"/>
-      <c r="UI2" s="50"/>
-      <c r="UJ2" s="50"/>
-      <c r="UK2" s="50"/>
-      <c r="UL2" s="50"/>
-      <c r="UM2" s="50"/>
-      <c r="UN2" s="50"/>
-      <c r="UO2" s="50"/>
-      <c r="UP2" s="50"/>
-      <c r="UQ2" s="50"/>
-      <c r="UR2" s="50"/>
-      <c r="US2" s="50"/>
-      <c r="UT2" s="50"/>
-      <c r="UU2" s="50"/>
-      <c r="UV2" s="50"/>
-      <c r="UW2" s="50"/>
-      <c r="UX2" s="50"/>
-      <c r="UY2" s="50"/>
-      <c r="UZ2" s="50"/>
-      <c r="VA2" s="50"/>
-      <c r="VB2" s="50"/>
-      <c r="VC2" s="50"/>
-      <c r="VD2" s="50"/>
-      <c r="VE2" s="50"/>
-      <c r="VF2" s="50"/>
-      <c r="VG2" s="50"/>
-      <c r="VH2" s="45" t="s">
+      <c r="TY2" s="47"/>
+      <c r="TZ2" s="47"/>
+      <c r="UA2" s="47"/>
+      <c r="UB2" s="47"/>
+      <c r="UC2" s="47"/>
+      <c r="UD2" s="47"/>
+      <c r="UE2" s="47"/>
+      <c r="UF2" s="47"/>
+      <c r="UG2" s="47"/>
+      <c r="UH2" s="47"/>
+      <c r="UI2" s="47"/>
+      <c r="UJ2" s="47"/>
+      <c r="UK2" s="47"/>
+      <c r="UL2" s="47"/>
+      <c r="UM2" s="47"/>
+      <c r="UN2" s="47"/>
+      <c r="UO2" s="47"/>
+      <c r="UP2" s="47"/>
+      <c r="UQ2" s="47"/>
+      <c r="UR2" s="47"/>
+      <c r="US2" s="47"/>
+      <c r="UT2" s="47"/>
+      <c r="UU2" s="47"/>
+      <c r="UV2" s="47"/>
+      <c r="UW2" s="47"/>
+      <c r="UX2" s="47"/>
+      <c r="UY2" s="47"/>
+      <c r="UZ2" s="47"/>
+      <c r="VA2" s="47"/>
+      <c r="VB2" s="47"/>
+      <c r="VC2" s="47"/>
+      <c r="VD2" s="47"/>
+      <c r="VE2" s="47"/>
+      <c r="VF2" s="47"/>
+      <c r="VG2" s="47"/>
+      <c r="VH2" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="VI2" s="45"/>
-      <c r="VJ2" s="45"/>
-      <c r="VK2" s="45"/>
-      <c r="VL2" s="45"/>
-      <c r="VM2" s="45"/>
-      <c r="VN2" s="45"/>
-      <c r="VO2" s="45"/>
-      <c r="VP2" s="45"/>
-      <c r="VQ2" s="45"/>
-      <c r="VR2" s="45"/>
-      <c r="VS2" s="45"/>
-      <c r="VT2" s="45"/>
-      <c r="VU2" s="45"/>
-      <c r="VV2" s="45"/>
-      <c r="VW2" s="45"/>
-      <c r="VX2" s="45"/>
-      <c r="VY2" s="45"/>
-      <c r="VZ2" s="45"/>
-      <c r="WA2" s="45"/>
-      <c r="WB2" s="45"/>
-      <c r="WC2" s="45"/>
-      <c r="WD2" s="45"/>
-      <c r="WE2" s="45"/>
-      <c r="WF2" s="45"/>
-      <c r="WG2" s="45"/>
-      <c r="WH2" s="45"/>
-      <c r="WI2" s="45"/>
-      <c r="WJ2" s="45"/>
-      <c r="WK2" s="45"/>
-      <c r="WL2" s="45"/>
+      <c r="VI2" s="41"/>
+      <c r="VJ2" s="41"/>
+      <c r="VK2" s="41"/>
+      <c r="VL2" s="41"/>
+      <c r="VM2" s="41"/>
+      <c r="VN2" s="41"/>
+      <c r="VO2" s="41"/>
+      <c r="VP2" s="41"/>
+      <c r="VQ2" s="41"/>
+      <c r="VR2" s="41"/>
+      <c r="VS2" s="41"/>
+      <c r="VT2" s="41"/>
+      <c r="VU2" s="41"/>
+      <c r="VV2" s="41"/>
+      <c r="VW2" s="41"/>
+      <c r="VX2" s="41"/>
+      <c r="VY2" s="41"/>
+      <c r="VZ2" s="41"/>
+      <c r="WA2" s="41"/>
+      <c r="WB2" s="41"/>
+      <c r="WC2" s="41"/>
+      <c r="WD2" s="41"/>
+      <c r="WE2" s="41"/>
+      <c r="WF2" s="41"/>
+      <c r="WG2" s="41"/>
+      <c r="WH2" s="41"/>
+      <c r="WI2" s="41"/>
+      <c r="WJ2" s="41"/>
+      <c r="WK2" s="41"/>
+      <c r="WL2" s="41"/>
     </row>
     <row r="3" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -7677,387 +7699,387 @@
       <c r="B3" t="s">
         <v>140</v>
       </c>
-      <c r="DY3" s="51" t="s">
+      <c r="DY3" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="DZ3" s="38" t="s">
+      <c r="DZ3" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="EA3" s="38"/>
-      <c r="EB3" s="38"/>
-      <c r="EC3" s="38"/>
-      <c r="EM3" s="40" t="s">
+      <c r="EA3" s="44"/>
+      <c r="EB3" s="44"/>
+      <c r="EC3" s="44"/>
+      <c r="EM3" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="EN3" s="40"/>
-      <c r="EO3" s="40"/>
-      <c r="EP3" s="48" t="s">
+      <c r="EN3" s="45"/>
+      <c r="EO3" s="45"/>
+      <c r="EP3" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="EQ3" s="41" t="s">
+      <c r="EQ3" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="ET3" s="44" t="s">
+      <c r="ET3" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="EU3" s="44"/>
-      <c r="EV3" s="44"/>
-      <c r="EW3" s="44"/>
-      <c r="EX3" s="52" t="s">
+      <c r="EU3" s="40"/>
+      <c r="EV3" s="40"/>
+      <c r="EW3" s="40"/>
+      <c r="EX3" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="EY3" s="52"/>
-      <c r="EZ3" s="52"/>
-      <c r="FA3" s="52"/>
-      <c r="FB3" s="44" t="s">
+      <c r="EY3" s="54"/>
+      <c r="EZ3" s="54"/>
+      <c r="FA3" s="54"/>
+      <c r="FB3" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="FC3" s="44"/>
-      <c r="FD3" s="44"/>
-      <c r="FE3" s="44"/>
-      <c r="FF3" s="44"/>
-      <c r="FG3" s="44"/>
-      <c r="FH3" s="44"/>
-      <c r="FI3" s="44"/>
-      <c r="FJ3" s="44" t="s">
+      <c r="FC3" s="40"/>
+      <c r="FD3" s="40"/>
+      <c r="FE3" s="40"/>
+      <c r="FF3" s="40"/>
+      <c r="FG3" s="40"/>
+      <c r="FH3" s="40"/>
+      <c r="FI3" s="40"/>
+      <c r="FJ3" s="40" t="s">
         <v>50</v>
       </c>
-      <c r="FK3" s="44"/>
-      <c r="FL3" s="44"/>
-      <c r="FM3" s="44"/>
-      <c r="FN3" s="44"/>
-      <c r="FO3" s="44"/>
-      <c r="FP3" s="44"/>
-      <c r="FQ3" s="44"/>
-      <c r="FR3" s="44"/>
-      <c r="FS3" s="44"/>
-      <c r="FT3" s="44"/>
-      <c r="FU3" s="44"/>
-      <c r="FV3" s="44"/>
-      <c r="FW3" s="44"/>
-      <c r="GS3" s="54" t="s">
+      <c r="FK3" s="40"/>
+      <c r="FL3" s="40"/>
+      <c r="FM3" s="40"/>
+      <c r="FN3" s="40"/>
+      <c r="FO3" s="40"/>
+      <c r="FP3" s="40"/>
+      <c r="FQ3" s="40"/>
+      <c r="FR3" s="40"/>
+      <c r="FS3" s="40"/>
+      <c r="FT3" s="40"/>
+      <c r="FU3" s="40"/>
+      <c r="FV3" s="40"/>
+      <c r="FW3" s="40"/>
+      <c r="GS3" s="51" t="s">
         <v>52</v>
       </c>
-      <c r="GT3" s="53"/>
-      <c r="GU3" s="54" t="s">
+      <c r="GT3" s="52"/>
+      <c r="GU3" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="GV3" s="54"/>
-      <c r="GW3" s="54"/>
-      <c r="GX3" s="54"/>
-      <c r="GY3" s="54"/>
-      <c r="GZ3" s="54"/>
-      <c r="HA3" s="54"/>
-      <c r="HB3" s="55" t="s">
+      <c r="GV3" s="51"/>
+      <c r="GW3" s="51"/>
+      <c r="GX3" s="51"/>
+      <c r="GY3" s="51"/>
+      <c r="GZ3" s="51"/>
+      <c r="HA3" s="51"/>
+      <c r="HB3" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="HE3" s="54" t="s">
+      <c r="HE3" s="51" t="s">
         <v>55</v>
       </c>
-      <c r="HF3" s="54"/>
-      <c r="HG3" s="56" t="s">
+      <c r="HF3" s="51"/>
+      <c r="HG3" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="HH3" s="38"/>
-      <c r="HI3" s="38"/>
-      <c r="HJ3" s="38"/>
-      <c r="HK3" s="38"/>
-      <c r="HL3" s="38"/>
-      <c r="HM3" s="45" t="s">
+      <c r="HH3" s="44"/>
+      <c r="HI3" s="44"/>
+      <c r="HJ3" s="44"/>
+      <c r="HK3" s="44"/>
+      <c r="HL3" s="44"/>
+      <c r="HM3" s="41" t="s">
         <v>58</v>
       </c>
-      <c r="HN3" s="45"/>
-      <c r="HO3" s="46" t="s">
+      <c r="HN3" s="41"/>
+      <c r="HO3" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="HP3" s="46"/>
-      <c r="HQ3" s="46"/>
-      <c r="HR3" s="46"/>
-      <c r="HS3" s="46"/>
-      <c r="HT3" s="46"/>
-      <c r="HU3" s="46"/>
-      <c r="HV3" s="46"/>
-      <c r="HW3" s="46"/>
-      <c r="HX3" s="46"/>
-      <c r="HY3" s="46"/>
-      <c r="HZ3" s="46"/>
-      <c r="IA3" s="46"/>
-      <c r="IB3" s="46"/>
-      <c r="IC3" s="45" t="s">
+      <c r="HP3" s="42"/>
+      <c r="HQ3" s="42"/>
+      <c r="HR3" s="42"/>
+      <c r="HS3" s="42"/>
+      <c r="HT3" s="42"/>
+      <c r="HU3" s="42"/>
+      <c r="HV3" s="42"/>
+      <c r="HW3" s="42"/>
+      <c r="HX3" s="42"/>
+      <c r="HY3" s="42"/>
+      <c r="HZ3" s="42"/>
+      <c r="IA3" s="42"/>
+      <c r="IB3" s="42"/>
+      <c r="IC3" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="ID3" s="45"/>
-      <c r="IE3" s="45"/>
-      <c r="IF3" s="45"/>
-      <c r="IG3" s="45"/>
-      <c r="IH3" s="45"/>
-      <c r="II3" s="45"/>
-      <c r="IJ3" s="45"/>
-      <c r="IK3" s="47" t="s">
+      <c r="ID3" s="41"/>
+      <c r="IE3" s="41"/>
+      <c r="IF3" s="41"/>
+      <c r="IG3" s="41"/>
+      <c r="IH3" s="41"/>
+      <c r="II3" s="41"/>
+      <c r="IJ3" s="41"/>
+      <c r="IK3" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="IL3" s="47"/>
-      <c r="IM3" s="47"/>
-      <c r="IN3" s="47"/>
-      <c r="IO3" s="47"/>
-      <c r="IP3" s="47"/>
-      <c r="IQ3" s="47"/>
-      <c r="IR3" s="40" t="s">
+      <c r="IL3" s="43"/>
+      <c r="IM3" s="43"/>
+      <c r="IN3" s="43"/>
+      <c r="IO3" s="43"/>
+      <c r="IP3" s="43"/>
+      <c r="IQ3" s="43"/>
+      <c r="IR3" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="IS3" s="40"/>
-      <c r="IT3" s="40"/>
-      <c r="IU3" s="40"/>
-      <c r="IV3" s="40"/>
-      <c r="IW3" s="46" t="s">
+      <c r="IS3" s="45"/>
+      <c r="IT3" s="45"/>
+      <c r="IU3" s="45"/>
+      <c r="IV3" s="45"/>
+      <c r="IW3" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="IX3" s="46"/>
-      <c r="IY3" s="46"/>
-      <c r="IZ3" s="46"/>
-      <c r="JA3" s="46"/>
-      <c r="JB3" s="46"/>
-      <c r="JC3" s="46"/>
-      <c r="JD3" s="46"/>
-      <c r="JE3" s="46"/>
-      <c r="JF3" s="46"/>
-      <c r="JG3" s="46"/>
-      <c r="JH3" s="46"/>
-      <c r="JI3" s="46"/>
-      <c r="JJ3" s="46"/>
-      <c r="JK3" s="46"/>
-      <c r="JL3" s="46"/>
-      <c r="JM3" s="46"/>
-      <c r="JN3" s="46"/>
-      <c r="JO3" s="46"/>
-      <c r="JP3" s="46"/>
-      <c r="JQ3" s="46"/>
-      <c r="JR3" s="46"/>
-      <c r="JS3" s="46"/>
-      <c r="JT3" s="46"/>
-      <c r="JU3" s="46"/>
-      <c r="JV3" s="46"/>
-      <c r="JW3" s="46"/>
-      <c r="JX3" s="46"/>
-      <c r="JY3" s="46"/>
-      <c r="JZ3" s="46"/>
-      <c r="KA3" s="46"/>
-      <c r="KB3" s="46"/>
-      <c r="KC3" s="46"/>
-      <c r="KD3" s="46"/>
-      <c r="KE3" s="46"/>
-      <c r="KF3" s="46"/>
-      <c r="KG3" s="46"/>
-      <c r="KH3" s="46"/>
-      <c r="KI3" s="46"/>
-      <c r="KJ3" s="46"/>
-      <c r="KK3" s="46"/>
-      <c r="KL3" s="46"/>
-      <c r="KM3" s="46"/>
-      <c r="KN3" s="46"/>
-      <c r="KO3" s="46"/>
-      <c r="KP3" s="46"/>
-      <c r="KQ3" s="46"/>
-      <c r="KR3" s="46"/>
-      <c r="KS3" s="59" t="s">
+      <c r="IX3" s="42"/>
+      <c r="IY3" s="42"/>
+      <c r="IZ3" s="42"/>
+      <c r="JA3" s="42"/>
+      <c r="JB3" s="42"/>
+      <c r="JC3" s="42"/>
+      <c r="JD3" s="42"/>
+      <c r="JE3" s="42"/>
+      <c r="JF3" s="42"/>
+      <c r="JG3" s="42"/>
+      <c r="JH3" s="42"/>
+      <c r="JI3" s="42"/>
+      <c r="JJ3" s="42"/>
+      <c r="JK3" s="42"/>
+      <c r="JL3" s="42"/>
+      <c r="JM3" s="42"/>
+      <c r="JN3" s="42"/>
+      <c r="JO3" s="42"/>
+      <c r="JP3" s="42"/>
+      <c r="JQ3" s="42"/>
+      <c r="JR3" s="42"/>
+      <c r="JS3" s="42"/>
+      <c r="JT3" s="42"/>
+      <c r="JU3" s="42"/>
+      <c r="JV3" s="42"/>
+      <c r="JW3" s="42"/>
+      <c r="JX3" s="42"/>
+      <c r="JY3" s="42"/>
+      <c r="JZ3" s="42"/>
+      <c r="KA3" s="42"/>
+      <c r="KB3" s="42"/>
+      <c r="KC3" s="42"/>
+      <c r="KD3" s="42"/>
+      <c r="KE3" s="42"/>
+      <c r="KF3" s="42"/>
+      <c r="KG3" s="42"/>
+      <c r="KH3" s="42"/>
+      <c r="KI3" s="42"/>
+      <c r="KJ3" s="42"/>
+      <c r="KK3" s="42"/>
+      <c r="KL3" s="42"/>
+      <c r="KM3" s="42"/>
+      <c r="KN3" s="42"/>
+      <c r="KO3" s="42"/>
+      <c r="KP3" s="42"/>
+      <c r="KQ3" s="42"/>
+      <c r="KR3" s="42"/>
+      <c r="KS3" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="KT3" s="59"/>
-      <c r="KU3" s="59"/>
-      <c r="KV3" s="59"/>
-      <c r="KW3" s="59"/>
-      <c r="KX3" s="59"/>
-      <c r="KY3" s="59"/>
-      <c r="KZ3" s="59"/>
-      <c r="LA3" s="59"/>
-      <c r="LB3" s="59"/>
-      <c r="LC3" s="59"/>
-      <c r="LD3" s="59"/>
-      <c r="LE3" s="59"/>
-      <c r="LF3" s="59"/>
-      <c r="LG3" s="59"/>
-      <c r="LH3" s="59"/>
-      <c r="LI3" s="59"/>
-      <c r="LJ3" s="59"/>
-      <c r="LK3" s="59"/>
-      <c r="LL3" s="59"/>
-      <c r="LM3" s="59"/>
-      <c r="LN3" s="59"/>
-      <c r="LO3" s="59"/>
-      <c r="LP3" s="59"/>
-      <c r="LQ3" s="59"/>
-      <c r="LR3" s="59"/>
-      <c r="LS3" s="59"/>
-      <c r="LT3" s="59"/>
-      <c r="LU3" s="59"/>
-      <c r="LV3" s="59"/>
-      <c r="LW3" s="59"/>
-      <c r="LX3" s="59"/>
-      <c r="MA3" s="59" t="s">
+      <c r="KT3" s="56"/>
+      <c r="KU3" s="56"/>
+      <c r="KV3" s="56"/>
+      <c r="KW3" s="56"/>
+      <c r="KX3" s="56"/>
+      <c r="KY3" s="56"/>
+      <c r="KZ3" s="56"/>
+      <c r="LA3" s="56"/>
+      <c r="LB3" s="56"/>
+      <c r="LC3" s="56"/>
+      <c r="LD3" s="56"/>
+      <c r="LE3" s="56"/>
+      <c r="LF3" s="56"/>
+      <c r="LG3" s="56"/>
+      <c r="LH3" s="56"/>
+      <c r="LI3" s="56"/>
+      <c r="LJ3" s="56"/>
+      <c r="LK3" s="56"/>
+      <c r="LL3" s="56"/>
+      <c r="LM3" s="56"/>
+      <c r="LN3" s="56"/>
+      <c r="LO3" s="56"/>
+      <c r="LP3" s="56"/>
+      <c r="LQ3" s="56"/>
+      <c r="LR3" s="56"/>
+      <c r="LS3" s="56"/>
+      <c r="LT3" s="56"/>
+      <c r="LU3" s="56"/>
+      <c r="LV3" s="56"/>
+      <c r="LW3" s="56"/>
+      <c r="LX3" s="56"/>
+      <c r="MA3" s="56" t="s">
         <v>66</v>
       </c>
-      <c r="MB3" s="59"/>
-      <c r="MC3" s="59"/>
-      <c r="MD3" s="59"/>
-      <c r="ME3" s="59"/>
-      <c r="MF3" s="59"/>
-      <c r="MG3" s="59"/>
-      <c r="MH3" s="59"/>
-      <c r="MI3" s="59"/>
-      <c r="MJ3" s="59"/>
-      <c r="MK3" s="59"/>
-      <c r="ML3" s="47" t="s">
+      <c r="MB3" s="56"/>
+      <c r="MC3" s="56"/>
+      <c r="MD3" s="56"/>
+      <c r="ME3" s="56"/>
+      <c r="MF3" s="56"/>
+      <c r="MG3" s="56"/>
+      <c r="MH3" s="56"/>
+      <c r="MI3" s="56"/>
+      <c r="MJ3" s="56"/>
+      <c r="MK3" s="56"/>
+      <c r="ML3" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="MM3" s="47"/>
-      <c r="MN3" s="47"/>
-      <c r="MO3" s="47"/>
-      <c r="MP3" s="47"/>
-      <c r="MQ3" s="47"/>
-      <c r="MR3" s="47"/>
-      <c r="MS3" s="47"/>
-      <c r="MT3" s="47"/>
-      <c r="MU3" s="47"/>
-      <c r="MV3" s="47"/>
-      <c r="MW3" s="47"/>
-      <c r="MX3" s="47"/>
-      <c r="MY3" s="47"/>
-      <c r="MZ3" s="47"/>
-      <c r="NA3" s="47"/>
-      <c r="NB3" s="47"/>
-      <c r="NC3" s="47"/>
-      <c r="ND3" s="47"/>
-      <c r="NE3" s="47"/>
-      <c r="NF3" s="47"/>
-      <c r="NG3" s="47"/>
-      <c r="NH3" s="47"/>
-      <c r="NI3" s="47"/>
-      <c r="NJ3" s="47"/>
-      <c r="NK3" s="47"/>
-      <c r="NL3" s="47"/>
-      <c r="NM3" s="47"/>
-      <c r="NN3" s="47"/>
-      <c r="NQ3" s="39" t="s">
+      <c r="MM3" s="43"/>
+      <c r="MN3" s="43"/>
+      <c r="MO3" s="43"/>
+      <c r="MP3" s="43"/>
+      <c r="MQ3" s="43"/>
+      <c r="MR3" s="43"/>
+      <c r="MS3" s="43"/>
+      <c r="MT3" s="43"/>
+      <c r="MU3" s="43"/>
+      <c r="MV3" s="43"/>
+      <c r="MW3" s="43"/>
+      <c r="MX3" s="43"/>
+      <c r="MY3" s="43"/>
+      <c r="MZ3" s="43"/>
+      <c r="NA3" s="43"/>
+      <c r="NB3" s="43"/>
+      <c r="NC3" s="43"/>
+      <c r="ND3" s="43"/>
+      <c r="NE3" s="43"/>
+      <c r="NF3" s="43"/>
+      <c r="NG3" s="43"/>
+      <c r="NH3" s="43"/>
+      <c r="NI3" s="43"/>
+      <c r="NJ3" s="43"/>
+      <c r="NK3" s="43"/>
+      <c r="NL3" s="43"/>
+      <c r="NM3" s="43"/>
+      <c r="NN3" s="43"/>
+      <c r="NQ3" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="NR3" s="40"/>
-      <c r="NS3" s="40"/>
-      <c r="NT3" s="40"/>
-      <c r="NU3" s="40"/>
-      <c r="NV3" s="40"/>
-      <c r="NW3" s="40"/>
-      <c r="NX3" s="40"/>
-      <c r="NY3" s="40"/>
-      <c r="NZ3" s="40"/>
-      <c r="OA3" s="40"/>
-      <c r="OB3" s="40"/>
-      <c r="OC3" s="40"/>
-      <c r="OD3" s="40"/>
-      <c r="OE3" s="40"/>
-      <c r="OF3" s="40"/>
-      <c r="OH3" s="38" t="s">
+      <c r="NR3" s="45"/>
+      <c r="NS3" s="45"/>
+      <c r="NT3" s="45"/>
+      <c r="NU3" s="45"/>
+      <c r="NV3" s="45"/>
+      <c r="NW3" s="45"/>
+      <c r="NX3" s="45"/>
+      <c r="NY3" s="45"/>
+      <c r="NZ3" s="45"/>
+      <c r="OA3" s="45"/>
+      <c r="OB3" s="45"/>
+      <c r="OC3" s="45"/>
+      <c r="OD3" s="45"/>
+      <c r="OE3" s="45"/>
+      <c r="OF3" s="45"/>
+      <c r="OH3" s="44" t="s">
         <v>70</v>
       </c>
-      <c r="OI3" s="38"/>
-      <c r="OJ3" s="38"/>
-      <c r="OK3" s="38"/>
-      <c r="OL3" s="38"/>
-      <c r="OM3" s="38"/>
-      <c r="ON3" s="38"/>
-      <c r="OO3" s="38"/>
-      <c r="OP3" s="38"/>
-      <c r="OQ3" s="38"/>
-      <c r="OR3" s="38"/>
-      <c r="OS3" s="38"/>
-      <c r="OT3" s="60" t="s">
+      <c r="OI3" s="44"/>
+      <c r="OJ3" s="44"/>
+      <c r="OK3" s="44"/>
+      <c r="OL3" s="44"/>
+      <c r="OM3" s="44"/>
+      <c r="ON3" s="44"/>
+      <c r="OO3" s="44"/>
+      <c r="OP3" s="44"/>
+      <c r="OQ3" s="44"/>
+      <c r="OR3" s="44"/>
+      <c r="OS3" s="44"/>
+      <c r="OT3" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="OU3" s="59" t="s">
+      <c r="OU3" s="56" t="s">
         <v>72</v>
       </c>
-      <c r="OV3" s="59"/>
-      <c r="OW3" s="59"/>
-      <c r="OX3" s="59"/>
-      <c r="OY3" s="59"/>
-      <c r="OZ3" s="59"/>
-      <c r="PA3" s="59"/>
-      <c r="PB3" s="59"/>
-      <c r="PC3" s="59"/>
-      <c r="PD3" s="59"/>
-      <c r="PE3" s="59"/>
-      <c r="PF3" s="59"/>
-      <c r="PG3" s="59"/>
-      <c r="PH3" s="59"/>
-      <c r="PI3" s="59"/>
-      <c r="PJ3" s="59"/>
-      <c r="PK3" s="59"/>
-      <c r="PL3" s="59"/>
-      <c r="PM3" s="59"/>
-      <c r="PN3" s="59"/>
-      <c r="PO3" s="59"/>
-      <c r="PP3" s="59"/>
-      <c r="PQ3" s="59"/>
-      <c r="PR3" s="45" t="s">
+      <c r="OV3" s="56"/>
+      <c r="OW3" s="56"/>
+      <c r="OX3" s="56"/>
+      <c r="OY3" s="56"/>
+      <c r="OZ3" s="56"/>
+      <c r="PA3" s="56"/>
+      <c r="PB3" s="56"/>
+      <c r="PC3" s="56"/>
+      <c r="PD3" s="56"/>
+      <c r="PE3" s="56"/>
+      <c r="PF3" s="56"/>
+      <c r="PG3" s="56"/>
+      <c r="PH3" s="56"/>
+      <c r="PI3" s="56"/>
+      <c r="PJ3" s="56"/>
+      <c r="PK3" s="56"/>
+      <c r="PL3" s="56"/>
+      <c r="PM3" s="56"/>
+      <c r="PN3" s="56"/>
+      <c r="PO3" s="56"/>
+      <c r="PP3" s="56"/>
+      <c r="PQ3" s="56"/>
+      <c r="PR3" s="41" t="s">
         <v>73</v>
       </c>
-      <c r="PS3" s="45"/>
-      <c r="PT3" s="45"/>
-      <c r="PU3" s="45"/>
-      <c r="PV3" s="45"/>
-      <c r="PW3" s="45"/>
-      <c r="PX3" s="45"/>
-      <c r="PY3" s="45"/>
-      <c r="PZ3" s="45"/>
-      <c r="QA3" s="45"/>
-      <c r="QB3" s="45"/>
-      <c r="QC3" s="45"/>
-      <c r="QD3" s="45"/>
-      <c r="QE3" s="45"/>
-      <c r="QF3" s="45"/>
-      <c r="QG3" s="45"/>
-      <c r="QH3" s="45"/>
-      <c r="QI3" s="45"/>
-      <c r="QJ3" s="45"/>
-      <c r="RY3" s="50" t="s">
+      <c r="PS3" s="41"/>
+      <c r="PT3" s="41"/>
+      <c r="PU3" s="41"/>
+      <c r="PV3" s="41"/>
+      <c r="PW3" s="41"/>
+      <c r="PX3" s="41"/>
+      <c r="PY3" s="41"/>
+      <c r="PZ3" s="41"/>
+      <c r="QA3" s="41"/>
+      <c r="QB3" s="41"/>
+      <c r="QC3" s="41"/>
+      <c r="QD3" s="41"/>
+      <c r="QE3" s="41"/>
+      <c r="QF3" s="41"/>
+      <c r="QG3" s="41"/>
+      <c r="QH3" s="41"/>
+      <c r="QI3" s="41"/>
+      <c r="QJ3" s="41"/>
+      <c r="RY3" s="47" t="s">
         <v>74</v>
       </c>
-      <c r="RZ3" s="50"/>
-      <c r="SA3" s="50"/>
-      <c r="SB3" s="50"/>
-      <c r="SC3" s="50"/>
-      <c r="SD3" s="50"/>
-      <c r="SE3" s="50"/>
-      <c r="SF3" s="50"/>
-      <c r="SG3" s="50"/>
-      <c r="SH3" s="50"/>
-      <c r="SI3" s="50"/>
-      <c r="SJ3" s="50"/>
-      <c r="SK3" s="50"/>
-      <c r="SL3" s="50"/>
-      <c r="SM3" s="50"/>
-      <c r="SN3" s="50"/>
-      <c r="SO3" s="50"/>
-      <c r="SP3" s="50"/>
-      <c r="SQ3" s="50"/>
-      <c r="SR3" s="50"/>
-      <c r="SS3" s="50"/>
-      <c r="ST3" s="50"/>
-      <c r="SU3" s="50"/>
-      <c r="SV3" s="50"/>
-      <c r="SW3" s="50"/>
-      <c r="SX3" s="50"/>
-      <c r="SY3" s="50"/>
-      <c r="SZ3" s="50"/>
-      <c r="TA3" s="50"/>
-      <c r="TB3" s="50"/>
-      <c r="TC3" s="50"/>
-      <c r="TD3" s="50"/>
-      <c r="TE3" s="50"/>
-      <c r="TF3" s="50"/>
-      <c r="TG3" s="50"/>
-      <c r="TH3" s="50"/>
-      <c r="TI3" s="50"/>
-      <c r="TJ3" s="50"/>
+      <c r="RZ3" s="47"/>
+      <c r="SA3" s="47"/>
+      <c r="SB3" s="47"/>
+      <c r="SC3" s="47"/>
+      <c r="SD3" s="47"/>
+      <c r="SE3" s="47"/>
+      <c r="SF3" s="47"/>
+      <c r="SG3" s="47"/>
+      <c r="SH3" s="47"/>
+      <c r="SI3" s="47"/>
+      <c r="SJ3" s="47"/>
+      <c r="SK3" s="47"/>
+      <c r="SL3" s="47"/>
+      <c r="SM3" s="47"/>
+      <c r="SN3" s="47"/>
+      <c r="SO3" s="47"/>
+      <c r="SP3" s="47"/>
+      <c r="SQ3" s="47"/>
+      <c r="SR3" s="47"/>
+      <c r="SS3" s="47"/>
+      <c r="ST3" s="47"/>
+      <c r="SU3" s="47"/>
+      <c r="SV3" s="47"/>
+      <c r="SW3" s="47"/>
+      <c r="SX3" s="47"/>
+      <c r="SY3" s="47"/>
+      <c r="SZ3" s="47"/>
+      <c r="TA3" s="47"/>
+      <c r="TB3" s="47"/>
+      <c r="TC3" s="47"/>
+      <c r="TD3" s="47"/>
+      <c r="TE3" s="47"/>
+      <c r="TF3" s="47"/>
+      <c r="TG3" s="47"/>
+      <c r="TH3" s="47"/>
+      <c r="TI3" s="47"/>
+      <c r="TJ3" s="47"/>
     </row>
     <row r="4" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -8066,17 +8088,17 @@
       <c r="B4" t="s">
         <v>141</v>
       </c>
-      <c r="HG4" s="51" t="s">
+      <c r="HG4" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="HH4" s="38" t="s">
+      <c r="HH4" s="44" t="s">
         <v>77</v>
       </c>
-      <c r="HI4" s="38"/>
-      <c r="HJ4" s="38"/>
-      <c r="HK4" s="38"/>
-      <c r="HL4" s="38"/>
-      <c r="HM4" s="38"/>
+      <c r="HI4" s="44"/>
+      <c r="HJ4" s="44"/>
+      <c r="HK4" s="44"/>
+      <c r="HL4" s="44"/>
+      <c r="HM4" s="44"/>
     </row>
     <row r="5" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -8085,30 +8107,30 @@
       <c r="B5" t="s">
         <v>130</v>
       </c>
-      <c r="HN5" s="38" t="s">
+      <c r="HN5" s="44" t="s">
         <v>79</v>
       </c>
-      <c r="HO5" s="38"/>
-      <c r="HP5" s="38"/>
-      <c r="HQ5" s="38"/>
-      <c r="HR5" s="38"/>
-      <c r="HS5" s="38"/>
-      <c r="HT5" s="38"/>
-      <c r="HU5" s="38"/>
-      <c r="HV5" s="38"/>
-      <c r="HW5" s="38"/>
-      <c r="HX5" s="38"/>
-      <c r="HY5" s="38"/>
-      <c r="HZ5" s="38"/>
-      <c r="IA5" s="38"/>
-      <c r="IB5" s="38"/>
-      <c r="IC5" s="38"/>
-      <c r="ID5" s="61" t="s">
+      <c r="HO5" s="44"/>
+      <c r="HP5" s="44"/>
+      <c r="HQ5" s="44"/>
+      <c r="HR5" s="44"/>
+      <c r="HS5" s="44"/>
+      <c r="HT5" s="44"/>
+      <c r="HU5" s="44"/>
+      <c r="HV5" s="44"/>
+      <c r="HW5" s="44"/>
+      <c r="HX5" s="44"/>
+      <c r="HY5" s="44"/>
+      <c r="HZ5" s="44"/>
+      <c r="IA5" s="44"/>
+      <c r="IB5" s="44"/>
+      <c r="IC5" s="44"/>
+      <c r="ID5" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="IE5" s="61"/>
-      <c r="IF5" s="61"/>
-      <c r="IG5" s="61"/>
+      <c r="IE5" s="55"/>
+      <c r="IF5" s="55"/>
+      <c r="IG5" s="55"/>
     </row>
     <row r="6" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -8117,28 +8139,28 @@
       <c r="B6" t="s">
         <v>131</v>
       </c>
-      <c r="IH6" s="38" t="s">
+      <c r="IH6" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="II6" s="38"/>
-      <c r="IJ6" s="38"/>
-      <c r="IK6" s="38"/>
-      <c r="IL6" s="38"/>
-      <c r="IM6" s="38"/>
-      <c r="IN6" s="38"/>
-      <c r="IO6" s="38"/>
-      <c r="IP6" s="38"/>
-      <c r="IQ6" s="38"/>
-      <c r="IR6" s="38"/>
-      <c r="IS6" s="38"/>
-      <c r="IT6" s="38"/>
-      <c r="IU6" s="38"/>
-      <c r="IV6" s="38"/>
-      <c r="IW6" s="38"/>
-      <c r="IX6" s="61" t="s">
+      <c r="II6" s="44"/>
+      <c r="IJ6" s="44"/>
+      <c r="IK6" s="44"/>
+      <c r="IL6" s="44"/>
+      <c r="IM6" s="44"/>
+      <c r="IN6" s="44"/>
+      <c r="IO6" s="44"/>
+      <c r="IP6" s="44"/>
+      <c r="IQ6" s="44"/>
+      <c r="IR6" s="44"/>
+      <c r="IS6" s="44"/>
+      <c r="IT6" s="44"/>
+      <c r="IU6" s="44"/>
+      <c r="IV6" s="44"/>
+      <c r="IW6" s="44"/>
+      <c r="IX6" s="55" t="s">
         <v>84</v>
       </c>
-      <c r="IY6" s="61"/>
+      <c r="IY6" s="55"/>
     </row>
     <row r="7" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -8147,35 +8169,35 @@
       <c r="B7" t="s">
         <v>132</v>
       </c>
-      <c r="JB7" s="38" t="s">
+      <c r="JB7" s="44" t="s">
         <v>86</v>
       </c>
-      <c r="JC7" s="38"/>
-      <c r="JD7" s="38"/>
-      <c r="JE7" s="38"/>
-      <c r="JF7" s="38"/>
-      <c r="JG7" s="38"/>
-      <c r="JH7" s="38"/>
-      <c r="JI7" s="38"/>
-      <c r="JJ7" s="38"/>
-      <c r="JK7" s="38"/>
-      <c r="JL7" s="38"/>
-      <c r="JM7" s="38"/>
-      <c r="JN7" s="38"/>
-      <c r="JO7" s="38"/>
-      <c r="JP7" s="38"/>
-      <c r="JQ7" s="38"/>
-      <c r="JR7" s="38"/>
-      <c r="JS7" s="38"/>
-      <c r="JT7" s="38"/>
-      <c r="JU7" s="38"/>
-      <c r="JV7" s="38"/>
-      <c r="JW7" s="38"/>
-      <c r="JX7" s="38"/>
-      <c r="JY7" s="61" t="s">
+      <c r="JC7" s="44"/>
+      <c r="JD7" s="44"/>
+      <c r="JE7" s="44"/>
+      <c r="JF7" s="44"/>
+      <c r="JG7" s="44"/>
+      <c r="JH7" s="44"/>
+      <c r="JI7" s="44"/>
+      <c r="JJ7" s="44"/>
+      <c r="JK7" s="44"/>
+      <c r="JL7" s="44"/>
+      <c r="JM7" s="44"/>
+      <c r="JN7" s="44"/>
+      <c r="JO7" s="44"/>
+      <c r="JP7" s="44"/>
+      <c r="JQ7" s="44"/>
+      <c r="JR7" s="44"/>
+      <c r="JS7" s="44"/>
+      <c r="JT7" s="44"/>
+      <c r="JU7" s="44"/>
+      <c r="JV7" s="44"/>
+      <c r="JW7" s="44"/>
+      <c r="JX7" s="44"/>
+      <c r="JY7" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="JZ7" s="61"/>
+      <c r="JZ7" s="55"/>
     </row>
     <row r="8" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -8184,30 +8206,30 @@
       <c r="B8" t="s">
         <v>133</v>
       </c>
-      <c r="KA8" s="38" t="s">
+      <c r="KA8" s="44" t="s">
         <v>89</v>
       </c>
-      <c r="KB8" s="38"/>
-      <c r="KC8" s="38"/>
-      <c r="KD8" s="38"/>
-      <c r="KE8" s="38"/>
-      <c r="KF8" s="38"/>
-      <c r="KG8" s="38"/>
-      <c r="KH8" s="38"/>
-      <c r="KI8" s="38"/>
-      <c r="KJ8" s="38"/>
-      <c r="KK8" s="38"/>
-      <c r="KL8" s="38"/>
-      <c r="KM8" s="38"/>
-      <c r="KN8" s="38"/>
-      <c r="KO8" s="38"/>
-      <c r="KP8" s="38"/>
-      <c r="KQ8" s="38"/>
-      <c r="KR8" s="38"/>
-      <c r="KS8" s="61" t="s">
+      <c r="KB8" s="44"/>
+      <c r="KC8" s="44"/>
+      <c r="KD8" s="44"/>
+      <c r="KE8" s="44"/>
+      <c r="KF8" s="44"/>
+      <c r="KG8" s="44"/>
+      <c r="KH8" s="44"/>
+      <c r="KI8" s="44"/>
+      <c r="KJ8" s="44"/>
+      <c r="KK8" s="44"/>
+      <c r="KL8" s="44"/>
+      <c r="KM8" s="44"/>
+      <c r="KN8" s="44"/>
+      <c r="KO8" s="44"/>
+      <c r="KP8" s="44"/>
+      <c r="KQ8" s="44"/>
+      <c r="KR8" s="44"/>
+      <c r="KS8" s="55" t="s">
         <v>90</v>
       </c>
-      <c r="KT8" s="61"/>
+      <c r="KT8" s="55"/>
     </row>
     <row r="9" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -8216,59 +8238,59 @@
       <c r="B9" t="s">
         <v>134</v>
       </c>
-      <c r="KU9" s="38" t="s">
+      <c r="KU9" s="44" t="s">
         <v>92</v>
       </c>
-      <c r="KV9" s="38"/>
-      <c r="KW9" s="38"/>
-      <c r="KX9" s="38"/>
-      <c r="KY9" s="38"/>
-      <c r="KZ9" s="38"/>
-      <c r="LA9" s="38"/>
-      <c r="LB9" s="38"/>
-      <c r="LC9" s="38"/>
-      <c r="LD9" s="38"/>
-      <c r="LE9" s="38"/>
-      <c r="LF9" s="38"/>
-      <c r="LG9" s="38"/>
-      <c r="LH9" s="38"/>
-      <c r="LI9" s="38"/>
-      <c r="LJ9" s="38"/>
-      <c r="LM9" s="61" t="s">
+      <c r="KV9" s="44"/>
+      <c r="KW9" s="44"/>
+      <c r="KX9" s="44"/>
+      <c r="KY9" s="44"/>
+      <c r="KZ9" s="44"/>
+      <c r="LA9" s="44"/>
+      <c r="LB9" s="44"/>
+      <c r="LC9" s="44"/>
+      <c r="LD9" s="44"/>
+      <c r="LE9" s="44"/>
+      <c r="LF9" s="44"/>
+      <c r="LG9" s="44"/>
+      <c r="LH9" s="44"/>
+      <c r="LI9" s="44"/>
+      <c r="LJ9" s="44"/>
+      <c r="LM9" s="55" t="s">
         <v>93</v>
       </c>
-      <c r="LN9" s="61"/>
-      <c r="LO9" s="38" t="s">
+      <c r="LN9" s="55"/>
+      <c r="LO9" s="44" t="s">
         <v>94</v>
       </c>
-      <c r="LP9" s="38"/>
-      <c r="LQ9" s="38"/>
-      <c r="LR9" s="38"/>
-      <c r="LS9" s="38"/>
-      <c r="LT9" s="38"/>
-      <c r="LU9" s="61" t="s">
+      <c r="LP9" s="44"/>
+      <c r="LQ9" s="44"/>
+      <c r="LR9" s="44"/>
+      <c r="LS9" s="44"/>
+      <c r="LT9" s="44"/>
+      <c r="LU9" s="55" t="s">
         <v>95</v>
       </c>
-      <c r="LV9" s="61"/>
-      <c r="LW9" s="61"/>
-      <c r="LX9" s="61"/>
-      <c r="LY9" s="61"/>
-      <c r="LZ9" s="61"/>
-      <c r="MA9" s="61"/>
-      <c r="MB9" s="61"/>
-      <c r="MC9" s="61"/>
-      <c r="MD9" s="61"/>
-      <c r="ME9" s="61"/>
-      <c r="MF9" s="61"/>
-      <c r="MG9" s="61"/>
-      <c r="MH9" s="61"/>
-      <c r="MI9" s="61"/>
-      <c r="MJ9" s="61"/>
-      <c r="MK9" s="61"/>
-      <c r="ML9" s="61"/>
-      <c r="MM9" s="61"/>
-      <c r="MN9" s="61"/>
-      <c r="MO9" s="61"/>
+      <c r="LV9" s="55"/>
+      <c r="LW9" s="55"/>
+      <c r="LX9" s="55"/>
+      <c r="LY9" s="55"/>
+      <c r="LZ9" s="55"/>
+      <c r="MA9" s="55"/>
+      <c r="MB9" s="55"/>
+      <c r="MC9" s="55"/>
+      <c r="MD9" s="55"/>
+      <c r="ME9" s="55"/>
+      <c r="MF9" s="55"/>
+      <c r="MG9" s="55"/>
+      <c r="MH9" s="55"/>
+      <c r="MI9" s="55"/>
+      <c r="MJ9" s="55"/>
+      <c r="MK9" s="55"/>
+      <c r="ML9" s="55"/>
+      <c r="MM9" s="55"/>
+      <c r="MN9" s="55"/>
+      <c r="MO9" s="55"/>
     </row>
     <row r="10" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -8277,17 +8299,17 @@
       <c r="B10" t="s">
         <v>142</v>
       </c>
-      <c r="HG10" s="51" t="s">
+      <c r="HG10" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="HH10" s="38" t="s">
+      <c r="HH10" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="HI10" s="38"/>
-      <c r="HJ10" s="38"/>
-      <c r="HK10" s="38"/>
-      <c r="HL10" s="38"/>
-      <c r="HM10" s="38"/>
+      <c r="HI10" s="44"/>
+      <c r="HJ10" s="44"/>
+      <c r="HK10" s="44"/>
+      <c r="HL10" s="44"/>
+      <c r="HM10" s="44"/>
     </row>
     <row r="11" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -8296,30 +8318,30 @@
       <c r="B11" t="s">
         <v>136</v>
       </c>
-      <c r="HN11" s="38" t="s">
+      <c r="HN11" s="44" t="s">
         <v>100</v>
       </c>
-      <c r="HO11" s="38"/>
-      <c r="HP11" s="38"/>
-      <c r="HQ11" s="38"/>
-      <c r="HR11" s="38"/>
-      <c r="HS11" s="38"/>
-      <c r="HT11" s="38"/>
-      <c r="HU11" s="38"/>
-      <c r="HV11" s="38"/>
-      <c r="HW11" s="38"/>
-      <c r="HX11" s="38"/>
-      <c r="HY11" s="38"/>
-      <c r="HZ11" s="38"/>
-      <c r="IA11" s="38"/>
-      <c r="IB11" s="38"/>
-      <c r="IC11" s="38"/>
-      <c r="ID11" s="62" t="s">
+      <c r="HO11" s="44"/>
+      <c r="HP11" s="44"/>
+      <c r="HQ11" s="44"/>
+      <c r="HR11" s="44"/>
+      <c r="HS11" s="44"/>
+      <c r="HT11" s="44"/>
+      <c r="HU11" s="44"/>
+      <c r="HV11" s="44"/>
+      <c r="HW11" s="44"/>
+      <c r="HX11" s="44"/>
+      <c r="HY11" s="44"/>
+      <c r="HZ11" s="44"/>
+      <c r="IA11" s="44"/>
+      <c r="IB11" s="44"/>
+      <c r="IC11" s="44"/>
+      <c r="ID11" s="58" t="s">
         <v>102</v>
       </c>
-      <c r="IE11" s="62"/>
-      <c r="IF11" s="62"/>
-      <c r="IG11" s="62"/>
+      <c r="IE11" s="58"/>
+      <c r="IF11" s="58"/>
+      <c r="IG11" s="58"/>
     </row>
     <row r="12" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -8328,28 +8350,28 @@
       <c r="B12" t="s">
         <v>137</v>
       </c>
-      <c r="IH12" s="38" t="s">
+      <c r="IH12" s="44" t="s">
         <v>104</v>
       </c>
-      <c r="II12" s="38"/>
-      <c r="IJ12" s="38"/>
-      <c r="IK12" s="38"/>
-      <c r="IL12" s="38"/>
-      <c r="IM12" s="38"/>
-      <c r="IN12" s="38"/>
-      <c r="IO12" s="38"/>
-      <c r="IP12" s="38"/>
-      <c r="IQ12" s="38"/>
-      <c r="IR12" s="38"/>
-      <c r="IS12" s="38"/>
-      <c r="IT12" s="38"/>
-      <c r="IU12" s="38"/>
-      <c r="IV12" s="38"/>
-      <c r="IW12" s="38"/>
-      <c r="IX12" s="62" t="s">
+      <c r="II12" s="44"/>
+      <c r="IJ12" s="44"/>
+      <c r="IK12" s="44"/>
+      <c r="IL12" s="44"/>
+      <c r="IM12" s="44"/>
+      <c r="IN12" s="44"/>
+      <c r="IO12" s="44"/>
+      <c r="IP12" s="44"/>
+      <c r="IQ12" s="44"/>
+      <c r="IR12" s="44"/>
+      <c r="IS12" s="44"/>
+      <c r="IT12" s="44"/>
+      <c r="IU12" s="44"/>
+      <c r="IV12" s="44"/>
+      <c r="IW12" s="44"/>
+      <c r="IX12" s="58" t="s">
         <v>105</v>
       </c>
-      <c r="IY12" s="62"/>
+      <c r="IY12" s="58"/>
     </row>
     <row r="13" spans="1:737" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -8358,184 +8380,57 @@
       <c r="B13" t="s">
         <v>138</v>
       </c>
-      <c r="JB13" s="38" t="s">
+      <c r="JB13" s="44" t="s">
         <v>107</v>
       </c>
-      <c r="JC13" s="38"/>
-      <c r="JD13" s="38"/>
-      <c r="JE13" s="38"/>
-      <c r="JF13" s="38"/>
-      <c r="JG13" s="38"/>
-      <c r="JH13" s="38"/>
-      <c r="JI13" s="38"/>
-      <c r="JJ13" s="38"/>
-      <c r="JK13" s="38"/>
-      <c r="JL13" s="38"/>
-      <c r="JM13" s="38"/>
-      <c r="JN13" s="38"/>
-      <c r="JO13" s="38"/>
-      <c r="JP13" s="38"/>
-      <c r="JQ13" s="38"/>
-      <c r="JR13" s="38"/>
-      <c r="JS13" s="38"/>
-      <c r="JT13" s="38"/>
-      <c r="JU13" s="38"/>
-      <c r="JV13" s="38"/>
-      <c r="JW13" s="38"/>
-      <c r="JX13" s="38"/>
-      <c r="JY13" s="62" t="s">
+      <c r="JC13" s="44"/>
+      <c r="JD13" s="44"/>
+      <c r="JE13" s="44"/>
+      <c r="JF13" s="44"/>
+      <c r="JG13" s="44"/>
+      <c r="JH13" s="44"/>
+      <c r="JI13" s="44"/>
+      <c r="JJ13" s="44"/>
+      <c r="JK13" s="44"/>
+      <c r="JL13" s="44"/>
+      <c r="JM13" s="44"/>
+      <c r="JN13" s="44"/>
+      <c r="JO13" s="44"/>
+      <c r="JP13" s="44"/>
+      <c r="JQ13" s="44"/>
+      <c r="JR13" s="44"/>
+      <c r="JS13" s="44"/>
+      <c r="JT13" s="44"/>
+      <c r="JU13" s="44"/>
+      <c r="JV13" s="44"/>
+      <c r="JW13" s="44"/>
+      <c r="JX13" s="44"/>
+      <c r="JY13" s="58" t="s">
         <v>108</v>
       </c>
-      <c r="JZ13" s="62"/>
-      <c r="KA13" s="38" t="s">
+      <c r="JZ13" s="58"/>
+      <c r="KA13" s="44" t="s">
         <v>109</v>
       </c>
-      <c r="KB13" s="38"/>
-      <c r="KC13" s="38"/>
-      <c r="KD13" s="38"/>
-      <c r="KE13" s="38"/>
-      <c r="KF13" s="38"/>
+      <c r="KB13" s="44"/>
+      <c r="KC13" s="44"/>
+      <c r="KD13" s="44"/>
+      <c r="KE13" s="44"/>
+      <c r="KF13" s="44"/>
     </row>
     <row r="14" spans="1:737" ht="13.8" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="171">
-    <mergeCell ref="X1:AD1"/>
-    <mergeCell ref="AE1:AK1"/>
-    <mergeCell ref="AL1:AR1"/>
-    <mergeCell ref="AS1:AY1"/>
-    <mergeCell ref="AZ1:BF1"/>
-    <mergeCell ref="BG1:BM1"/>
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="J1:P1"/>
-    <mergeCell ref="Q1:W1"/>
-    <mergeCell ref="DD1:DJ1"/>
-    <mergeCell ref="DK1:DQ1"/>
-    <mergeCell ref="DR1:DX1"/>
-    <mergeCell ref="DY1:EE1"/>
-    <mergeCell ref="EF1:EL1"/>
-    <mergeCell ref="EM1:ES1"/>
-    <mergeCell ref="BN1:BT1"/>
-    <mergeCell ref="BU1:CA1"/>
-    <mergeCell ref="CB1:CH1"/>
-    <mergeCell ref="CI1:CO1"/>
-    <mergeCell ref="CP1:CV1"/>
-    <mergeCell ref="CW1:DC1"/>
-    <mergeCell ref="GJ1:GP1"/>
-    <mergeCell ref="GQ1:GW1"/>
-    <mergeCell ref="GX1:HD1"/>
-    <mergeCell ref="HE1:HK1"/>
-    <mergeCell ref="HL1:HR1"/>
-    <mergeCell ref="HS1:HY1"/>
-    <mergeCell ref="ET1:EZ1"/>
-    <mergeCell ref="FA1:FG1"/>
-    <mergeCell ref="FH1:FN1"/>
-    <mergeCell ref="FO1:FU1"/>
-    <mergeCell ref="FV1:GB1"/>
-    <mergeCell ref="GC1:GI1"/>
-    <mergeCell ref="JP1:JV1"/>
-    <mergeCell ref="JW1:KC1"/>
-    <mergeCell ref="KD1:KJ1"/>
-    <mergeCell ref="KK1:KQ1"/>
-    <mergeCell ref="KR1:KX1"/>
-    <mergeCell ref="KY1:LE1"/>
-    <mergeCell ref="HZ1:IF1"/>
-    <mergeCell ref="IG1:IM1"/>
-    <mergeCell ref="IN1:IT1"/>
-    <mergeCell ref="IU1:JA1"/>
-    <mergeCell ref="JB1:JH1"/>
-    <mergeCell ref="JI1:JO1"/>
-    <mergeCell ref="MV1:NB1"/>
-    <mergeCell ref="NC1:NI1"/>
-    <mergeCell ref="NJ1:NP1"/>
-    <mergeCell ref="NQ1:NW1"/>
-    <mergeCell ref="NX1:OD1"/>
-    <mergeCell ref="OE1:OK1"/>
-    <mergeCell ref="LF1:LL1"/>
-    <mergeCell ref="LM1:LS1"/>
-    <mergeCell ref="LT1:LZ1"/>
-    <mergeCell ref="MA1:MG1"/>
-    <mergeCell ref="MH1:MN1"/>
-    <mergeCell ref="MO1:MU1"/>
-    <mergeCell ref="QB1:QH1"/>
-    <mergeCell ref="QI1:QO1"/>
-    <mergeCell ref="QP1:QV1"/>
-    <mergeCell ref="QW1:RC1"/>
-    <mergeCell ref="RD1:RJ1"/>
-    <mergeCell ref="RK1:RQ1"/>
-    <mergeCell ref="OL1:OR1"/>
-    <mergeCell ref="OS1:OY1"/>
-    <mergeCell ref="OZ1:PF1"/>
-    <mergeCell ref="PG1:PM1"/>
-    <mergeCell ref="PN1:PT1"/>
-    <mergeCell ref="PU1:QA1"/>
-    <mergeCell ref="TH1:TN1"/>
-    <mergeCell ref="TO1:TU1"/>
-    <mergeCell ref="TV1:UB1"/>
-    <mergeCell ref="UC1:UI1"/>
-    <mergeCell ref="UJ1:UP1"/>
-    <mergeCell ref="UQ1:UW1"/>
-    <mergeCell ref="RR1:RX1"/>
-    <mergeCell ref="RY1:SE1"/>
-    <mergeCell ref="SF1:SL1"/>
-    <mergeCell ref="SM1:SS1"/>
-    <mergeCell ref="ST1:SZ1"/>
-    <mergeCell ref="TA1:TG1"/>
-    <mergeCell ref="WN1:WT1"/>
-    <mergeCell ref="WU1:XA1"/>
-    <mergeCell ref="XB1:XH1"/>
-    <mergeCell ref="XI1:XO1"/>
-    <mergeCell ref="XP1:XV1"/>
-    <mergeCell ref="XW1:YC1"/>
-    <mergeCell ref="UX1:VD1"/>
-    <mergeCell ref="VE1:VK1"/>
-    <mergeCell ref="VL1:VR1"/>
-    <mergeCell ref="VS1:VY1"/>
-    <mergeCell ref="VZ1:WF1"/>
-    <mergeCell ref="WG1:WM1"/>
-    <mergeCell ref="ZT1:ZZ1"/>
-    <mergeCell ref="AAA1:AAG1"/>
-    <mergeCell ref="AAH1:AAN1"/>
-    <mergeCell ref="AAO1:AAU1"/>
-    <mergeCell ref="AAV1:ABB1"/>
-    <mergeCell ref="ABC1:ABI1"/>
-    <mergeCell ref="YD1:YJ1"/>
-    <mergeCell ref="YK1:YQ1"/>
-    <mergeCell ref="YR1:YX1"/>
-    <mergeCell ref="YY1:ZE1"/>
-    <mergeCell ref="ZF1:ZL1"/>
-    <mergeCell ref="ZM1:ZS1"/>
-    <mergeCell ref="IY2:JB2"/>
-    <mergeCell ref="JC2:JK2"/>
-    <mergeCell ref="JL2:KK2"/>
-    <mergeCell ref="KL2:KT2"/>
-    <mergeCell ref="KU2:LN2"/>
-    <mergeCell ref="LO2:LW2"/>
-    <mergeCell ref="GS2:HM2"/>
-    <mergeCell ref="HN2:HT2"/>
-    <mergeCell ref="HV2:IB2"/>
-    <mergeCell ref="IC2:II2"/>
-    <mergeCell ref="IK2:IU2"/>
-    <mergeCell ref="IV2:IX2"/>
-    <mergeCell ref="QX2:RN2"/>
-    <mergeCell ref="RO2:RU2"/>
-    <mergeCell ref="RV2:RZ2"/>
-    <mergeCell ref="SA2:TW2"/>
-    <mergeCell ref="TX2:VG2"/>
-    <mergeCell ref="VH2:WL2"/>
-    <mergeCell ref="OO2:QP2"/>
-    <mergeCell ref="NG2:OB2"/>
-    <mergeCell ref="QQ2:QW2"/>
-    <mergeCell ref="GS3:GT3"/>
-    <mergeCell ref="GU3:HA3"/>
-    <mergeCell ref="HE3:HF3"/>
-    <mergeCell ref="HG3:HL3"/>
-    <mergeCell ref="HM3:HN3"/>
-    <mergeCell ref="DZ3:EC3"/>
-    <mergeCell ref="EM3:EO3"/>
-    <mergeCell ref="ET3:EW3"/>
-    <mergeCell ref="EX3:FA3"/>
-    <mergeCell ref="FB3:FI3"/>
-    <mergeCell ref="FJ3:FW3"/>
+    <mergeCell ref="JB13:JX13"/>
+    <mergeCell ref="JY13:JZ13"/>
+    <mergeCell ref="KA13:KF13"/>
+    <mergeCell ref="LO9:LT9"/>
+    <mergeCell ref="LU9:MO9"/>
+    <mergeCell ref="HH10:HM10"/>
+    <mergeCell ref="HN11:IC11"/>
+    <mergeCell ref="ID11:IG11"/>
+    <mergeCell ref="IH12:IW12"/>
+    <mergeCell ref="IX12:IY12"/>
     <mergeCell ref="JB7:JX7"/>
     <mergeCell ref="JY7:JZ7"/>
     <mergeCell ref="KA8:KR8"/>
@@ -8560,16 +8455,143 @@
     <mergeCell ref="IR3:IV3"/>
     <mergeCell ref="IW3:KR3"/>
     <mergeCell ref="KS3:LX3"/>
-    <mergeCell ref="JB13:JX13"/>
-    <mergeCell ref="JY13:JZ13"/>
-    <mergeCell ref="KA13:KF13"/>
-    <mergeCell ref="LO9:LT9"/>
-    <mergeCell ref="LU9:MO9"/>
-    <mergeCell ref="HH10:HM10"/>
-    <mergeCell ref="HN11:IC11"/>
-    <mergeCell ref="ID11:IG11"/>
-    <mergeCell ref="IH12:IW12"/>
-    <mergeCell ref="IX12:IY12"/>
+    <mergeCell ref="GS3:GT3"/>
+    <mergeCell ref="GU3:HA3"/>
+    <mergeCell ref="HE3:HF3"/>
+    <mergeCell ref="HG3:HL3"/>
+    <mergeCell ref="HM3:HN3"/>
+    <mergeCell ref="DZ3:EC3"/>
+    <mergeCell ref="EM3:EO3"/>
+    <mergeCell ref="ET3:EW3"/>
+    <mergeCell ref="EX3:FA3"/>
+    <mergeCell ref="FB3:FI3"/>
+    <mergeCell ref="FJ3:FW3"/>
+    <mergeCell ref="QX2:RN2"/>
+    <mergeCell ref="RO2:RU2"/>
+    <mergeCell ref="RV2:RZ2"/>
+    <mergeCell ref="SA2:TW2"/>
+    <mergeCell ref="TX2:VG2"/>
+    <mergeCell ref="VH2:WL2"/>
+    <mergeCell ref="OO2:QP2"/>
+    <mergeCell ref="NG2:OB2"/>
+    <mergeCell ref="QQ2:QW2"/>
+    <mergeCell ref="IY2:JB2"/>
+    <mergeCell ref="JC2:JK2"/>
+    <mergeCell ref="JL2:KK2"/>
+    <mergeCell ref="KL2:KT2"/>
+    <mergeCell ref="KU2:LN2"/>
+    <mergeCell ref="LO2:LW2"/>
+    <mergeCell ref="GS2:HM2"/>
+    <mergeCell ref="HN2:HT2"/>
+    <mergeCell ref="HV2:IB2"/>
+    <mergeCell ref="IC2:II2"/>
+    <mergeCell ref="IK2:IU2"/>
+    <mergeCell ref="IV2:IX2"/>
+    <mergeCell ref="ZT1:ZZ1"/>
+    <mergeCell ref="AAA1:AAG1"/>
+    <mergeCell ref="AAH1:AAN1"/>
+    <mergeCell ref="AAO1:AAU1"/>
+    <mergeCell ref="AAV1:ABB1"/>
+    <mergeCell ref="ABC1:ABI1"/>
+    <mergeCell ref="YD1:YJ1"/>
+    <mergeCell ref="YK1:YQ1"/>
+    <mergeCell ref="YR1:YX1"/>
+    <mergeCell ref="YY1:ZE1"/>
+    <mergeCell ref="ZF1:ZL1"/>
+    <mergeCell ref="ZM1:ZS1"/>
+    <mergeCell ref="WN1:WT1"/>
+    <mergeCell ref="WU1:XA1"/>
+    <mergeCell ref="XB1:XH1"/>
+    <mergeCell ref="XI1:XO1"/>
+    <mergeCell ref="XP1:XV1"/>
+    <mergeCell ref="XW1:YC1"/>
+    <mergeCell ref="UX1:VD1"/>
+    <mergeCell ref="VE1:VK1"/>
+    <mergeCell ref="VL1:VR1"/>
+    <mergeCell ref="VS1:VY1"/>
+    <mergeCell ref="VZ1:WF1"/>
+    <mergeCell ref="WG1:WM1"/>
+    <mergeCell ref="TH1:TN1"/>
+    <mergeCell ref="TO1:TU1"/>
+    <mergeCell ref="TV1:UB1"/>
+    <mergeCell ref="UC1:UI1"/>
+    <mergeCell ref="UJ1:UP1"/>
+    <mergeCell ref="UQ1:UW1"/>
+    <mergeCell ref="RR1:RX1"/>
+    <mergeCell ref="RY1:SE1"/>
+    <mergeCell ref="SF1:SL1"/>
+    <mergeCell ref="SM1:SS1"/>
+    <mergeCell ref="ST1:SZ1"/>
+    <mergeCell ref="TA1:TG1"/>
+    <mergeCell ref="QB1:QH1"/>
+    <mergeCell ref="QI1:QO1"/>
+    <mergeCell ref="QP1:QV1"/>
+    <mergeCell ref="QW1:RC1"/>
+    <mergeCell ref="RD1:RJ1"/>
+    <mergeCell ref="RK1:RQ1"/>
+    <mergeCell ref="OL1:OR1"/>
+    <mergeCell ref="OS1:OY1"/>
+    <mergeCell ref="OZ1:PF1"/>
+    <mergeCell ref="PG1:PM1"/>
+    <mergeCell ref="PN1:PT1"/>
+    <mergeCell ref="PU1:QA1"/>
+    <mergeCell ref="MV1:NB1"/>
+    <mergeCell ref="NC1:NI1"/>
+    <mergeCell ref="NJ1:NP1"/>
+    <mergeCell ref="NQ1:NW1"/>
+    <mergeCell ref="NX1:OD1"/>
+    <mergeCell ref="OE1:OK1"/>
+    <mergeCell ref="LF1:LL1"/>
+    <mergeCell ref="LM1:LS1"/>
+    <mergeCell ref="LT1:LZ1"/>
+    <mergeCell ref="MA1:MG1"/>
+    <mergeCell ref="MH1:MN1"/>
+    <mergeCell ref="MO1:MU1"/>
+    <mergeCell ref="JP1:JV1"/>
+    <mergeCell ref="JW1:KC1"/>
+    <mergeCell ref="KD1:KJ1"/>
+    <mergeCell ref="KK1:KQ1"/>
+    <mergeCell ref="KR1:KX1"/>
+    <mergeCell ref="KY1:LE1"/>
+    <mergeCell ref="HZ1:IF1"/>
+    <mergeCell ref="IG1:IM1"/>
+    <mergeCell ref="IN1:IT1"/>
+    <mergeCell ref="IU1:JA1"/>
+    <mergeCell ref="JB1:JH1"/>
+    <mergeCell ref="JI1:JO1"/>
+    <mergeCell ref="GJ1:GP1"/>
+    <mergeCell ref="GQ1:GW1"/>
+    <mergeCell ref="GX1:HD1"/>
+    <mergeCell ref="HE1:HK1"/>
+    <mergeCell ref="HL1:HR1"/>
+    <mergeCell ref="HS1:HY1"/>
+    <mergeCell ref="ET1:EZ1"/>
+    <mergeCell ref="FA1:FG1"/>
+    <mergeCell ref="FH1:FN1"/>
+    <mergeCell ref="FO1:FU1"/>
+    <mergeCell ref="FV1:GB1"/>
+    <mergeCell ref="GC1:GI1"/>
+    <mergeCell ref="DD1:DJ1"/>
+    <mergeCell ref="DK1:DQ1"/>
+    <mergeCell ref="DR1:DX1"/>
+    <mergeCell ref="DY1:EE1"/>
+    <mergeCell ref="EF1:EL1"/>
+    <mergeCell ref="EM1:ES1"/>
+    <mergeCell ref="BN1:BT1"/>
+    <mergeCell ref="BU1:CA1"/>
+    <mergeCell ref="CB1:CH1"/>
+    <mergeCell ref="CI1:CO1"/>
+    <mergeCell ref="CP1:CV1"/>
+    <mergeCell ref="CW1:DC1"/>
+    <mergeCell ref="X1:AD1"/>
+    <mergeCell ref="AE1:AK1"/>
+    <mergeCell ref="AL1:AR1"/>
+    <mergeCell ref="AS1:AY1"/>
+    <mergeCell ref="AZ1:BF1"/>
+    <mergeCell ref="BG1:BM1"/>
+    <mergeCell ref="C1:I1"/>
+    <mergeCell ref="J1:P1"/>
+    <mergeCell ref="Q1:W1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9021,70 +9043,70 @@
       <c r="ER1" t="s">
         <v>115</v>
       </c>
-      <c r="ET1" s="35" t="s">
+      <c r="ET1" s="61" t="s">
         <v>119</v>
       </c>
-      <c r="EU1" s="35"/>
-      <c r="EV1" s="35"/>
-      <c r="EW1" s="35"/>
-      <c r="EX1" s="35"/>
-      <c r="EY1" s="35"/>
-      <c r="EZ1" s="35"/>
-      <c r="FA1" s="35" t="s">
+      <c r="EU1" s="61"/>
+      <c r="EV1" s="61"/>
+      <c r="EW1" s="61"/>
+      <c r="EX1" s="61"/>
+      <c r="EY1" s="61"/>
+      <c r="EZ1" s="61"/>
+      <c r="FA1" s="61" t="s">
         <v>121</v>
       </c>
-      <c r="FB1" s="35"/>
-      <c r="FC1" s="35"/>
-      <c r="FD1" s="35"/>
-      <c r="FE1" s="35"/>
-      <c r="FF1" s="35"/>
-      <c r="FG1" s="35"/>
-      <c r="FH1" s="36" t="s">
+      <c r="FB1" s="61"/>
+      <c r="FC1" s="61"/>
+      <c r="FD1" s="61"/>
+      <c r="FE1" s="61"/>
+      <c r="FF1" s="61"/>
+      <c r="FG1" s="61"/>
+      <c r="FH1" s="62" t="s">
         <v>120</v>
       </c>
-      <c r="FI1" s="37"/>
-      <c r="FJ1" s="37"/>
-      <c r="FK1" s="37"/>
-      <c r="FL1" s="37"/>
-      <c r="FM1" s="37"/>
-      <c r="FN1" s="37"/>
-      <c r="FO1" s="36" t="e">
+      <c r="FI1" s="63"/>
+      <c r="FJ1" s="63"/>
+      <c r="FK1" s="63"/>
+      <c r="FL1" s="63"/>
+      <c r="FM1" s="63"/>
+      <c r="FN1" s="63"/>
+      <c r="FO1" s="62" t="e">
         <f>FH1+7</f>
         <v>#VALUE!</v>
       </c>
-      <c r="FP1" s="37"/>
-      <c r="FQ1" s="37"/>
-      <c r="FR1" s="37"/>
-      <c r="FS1" s="37"/>
-      <c r="FT1" s="37"/>
-      <c r="FU1" s="37"/>
-      <c r="FV1" s="36" t="s">
+      <c r="FP1" s="63"/>
+      <c r="FQ1" s="63"/>
+      <c r="FR1" s="63"/>
+      <c r="FS1" s="63"/>
+      <c r="FT1" s="63"/>
+      <c r="FU1" s="63"/>
+      <c r="FV1" s="62" t="s">
         <v>122</v>
       </c>
-      <c r="FW1" s="37"/>
-      <c r="FX1" s="37"/>
-      <c r="FY1" s="37"/>
-      <c r="FZ1" s="37"/>
-      <c r="GA1" s="37"/>
-      <c r="GB1" s="37"/>
-      <c r="GC1" s="36" t="s">
+      <c r="FW1" s="63"/>
+      <c r="FX1" s="63"/>
+      <c r="FY1" s="63"/>
+      <c r="FZ1" s="63"/>
+      <c r="GA1" s="63"/>
+      <c r="GB1" s="63"/>
+      <c r="GC1" s="62" t="s">
         <v>123</v>
       </c>
-      <c r="GD1" s="37"/>
-      <c r="GE1" s="37"/>
-      <c r="GF1" s="37"/>
-      <c r="GG1" s="37"/>
-      <c r="GH1" s="37"/>
-      <c r="GI1" s="37"/>
-      <c r="GJ1" s="33" t="s">
+      <c r="GD1" s="63"/>
+      <c r="GE1" s="63"/>
+      <c r="GF1" s="63"/>
+      <c r="GG1" s="63"/>
+      <c r="GH1" s="63"/>
+      <c r="GI1" s="63"/>
+      <c r="GJ1" s="59" t="s">
         <v>124</v>
       </c>
-      <c r="GK1" s="34"/>
-      <c r="GL1" s="34"/>
-      <c r="GM1" s="34"/>
-      <c r="GN1" s="34"/>
-      <c r="GO1" s="34"/>
-      <c r="GP1" s="34"/>
+      <c r="GK1" s="60"/>
+      <c r="GL1" s="60"/>
+      <c r="GM1" s="60"/>
+      <c r="GN1" s="60"/>
+      <c r="GO1" s="60"/>
+      <c r="GP1" s="60"/>
       <c r="GQ1" t="s">
         <v>117</v>
       </c>

</xml_diff>